<commit_message>
Modified header of GCS_to_s3_copy.py to include copying all 2015-2024 data to s3. Modified decision tree to make fire branch node codes end in 9, and updated LULUCF_state_node_lookup_table.xlsx.
</commit_message>
<xml_diff>
--- a/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
+++ b/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIS\git\AFOLU_GHG_flux_model\src\LULUCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F67D5006-79B2-4C68-A133-179BAD39E94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EEA2BDC-D595-4D86-A8F5-322A3E5634B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-9180" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="v030_20250430" sheetId="1" r:id="rId1"/>
+    <sheet name="v040_20250805" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="158">
   <si>
     <t>meaning</t>
   </si>
@@ -270,13 +271,253 @@
   </si>
   <si>
     <t>state_nodes_with_prefix</t>
+  </si>
+  <si>
+    <t>state_nodes_unpadded</t>
+  </si>
+  <si>
+    <t>Gain of oil palm (incl. SDPT oil palm)</t>
+  </si>
+  <si>
+    <t>Gain of non-oil palm planted trees</t>
+  </si>
+  <si>
+    <t>Gain of terrestrial natural forest</t>
+  </si>
+  <si>
+    <t>Gain of trees outside forests</t>
+  </si>
+  <si>
+    <t>Full loss of oil palm (incl. SDPT) with fire</t>
+  </si>
+  <si>
+    <t>Full loss of oil palm (incl. SDPT) without fire</t>
+  </si>
+  <si>
+    <t>Full loss of non-oil palm tree crops as cropland with fire</t>
+  </si>
+  <si>
+    <t>Full loss of non-oil palm tree crops as cropland without fire</t>
+  </si>
+  <si>
+    <t>Full loss of non-oil palm planted forest as cropland with fire</t>
+  </si>
+  <si>
+    <t>Full loss of non-oil palm planted forest as cropland without fire</t>
+  </si>
+  <si>
+    <t>Full loss of non-oil palm tree crops as short vegetation with fire</t>
+  </si>
+  <si>
+    <t>Full loss of non-oil palm tree crops as short vegetation without fire</t>
+  </si>
+  <si>
+    <t>Full loss of non-oil palm planted forest as short vegetation with fire</t>
+  </si>
+  <si>
+    <t>Full loss of non-oil palm planted forest as short vegetation without fire</t>
+  </si>
+  <si>
+    <t>Full loss of non-oil palm tree crops to settlement with fire</t>
+  </si>
+  <si>
+    <t>Full loss of non-oil palm tree crops to settlement without fire</t>
+  </si>
+  <si>
+    <t>Full loss of non-oil palm planted forest to settlement with fire</t>
+  </si>
+  <si>
+    <t>Full loss of non-oil palm planted forest to settlement without fire</t>
+  </si>
+  <si>
+    <t>Full loss of non-oil palm tree crops to anything else without fire</t>
+  </si>
+  <si>
+    <t>Full loss of non-oil palm planted forest to anything else without fire</t>
+  </si>
+  <si>
+    <t>Natural forest converted to cropland with fire</t>
+  </si>
+  <si>
+    <t>Natural forest converted to cropland without fire</t>
+  </si>
+  <si>
+    <t>Natural forest converted to short vegetation with disturbance that emits all non-soil C pools with fire</t>
+  </si>
+  <si>
+    <t>Natural forest converted to short vegetation with disturbance that emits all non-soil C pools without fire</t>
+  </si>
+  <si>
+    <t>Natural forest converted to short vegetation with disturbance that emits biomass C pools only with fire</t>
+  </si>
+  <si>
+    <t>Natural forest converted to short vegetation with disturbance that emits biomass C pools only without fire</t>
+  </si>
+  <si>
+    <t>Natural forest converted to settlement with fire</t>
+  </si>
+  <si>
+    <t>Natural forest converted to settlement without fire</t>
+  </si>
+  <si>
+    <t>Natural forest converted to anything else (wetland/open water/ice, etc.) without fire</t>
+  </si>
+  <si>
+    <t>Full loss of trees outside forests converted to cropland with fire</t>
+  </si>
+  <si>
+    <t>Full loss of trees outside forests converted to cropland without fire</t>
+  </si>
+  <si>
+    <t>Full loss of trees outside forests converted to short vegetation with fire</t>
+  </si>
+  <si>
+    <t>Full loss of trees outside forests converted to short vegetation without fire</t>
+  </si>
+  <si>
+    <t>Full loss of trees outside forests converted to settlement with fire</t>
+  </si>
+  <si>
+    <t>Full loss of trees outside forests converted to settlement without fire</t>
+  </si>
+  <si>
+    <t>Full loss of trees outside forests converted to anything else without fire</t>
+  </si>
+  <si>
+    <t>Non-planted trees with oil palm planted in the next interval with fire</t>
+  </si>
+  <si>
+    <t>Non-planted trees with oil palm planted in the next interval without fire</t>
+  </si>
+  <si>
+    <t>Oil palm partially disturbed in the current interval with signif. height increase after with fire</t>
+  </si>
+  <si>
+    <t>Oil palm partially disturbed in the current interval with signif. height increase after without fire</t>
+  </si>
+  <si>
+    <t>Planted trees partially disturbed in the current interval with signif. height increase after with fire</t>
+  </si>
+  <si>
+    <t>Planted trees partially disturbed in the current interval with signif. height increase after without fire</t>
+  </si>
+  <si>
+    <t>Oil palm partially disturbed in the current interval without signif. height increase after with fire</t>
+  </si>
+  <si>
+    <t>Oil palm partially disturbed in the current interval without signif. height increase after without fire</t>
+  </si>
+  <si>
+    <t>Planted trees partially disturbed in the current interval without signif. height increase after with fire</t>
+  </si>
+  <si>
+    <t>Planted trees partially disturbed in the current interval without signif. height increase after without fire</t>
+  </si>
+  <si>
+    <t>Forest partially disturbed in the current interval with signif. height increase after with fire</t>
+  </si>
+  <si>
+    <t>Forest partially disturbed in the current interval with signif. height increase after without fire</t>
+  </si>
+  <si>
+    <t>Forest partially disturbed in the current interval without signif. height increase after with fire</t>
+  </si>
+  <si>
+    <t>Forest partially disturbed in the current interval without signif. height increase after without fire</t>
+  </si>
+  <si>
+    <t>Trees outside forests partially disturbed in the current interval with signif. height increase after with fire</t>
+  </si>
+  <si>
+    <t>Trees outside forests partially disturbed in the current interval with signif. height increase after without fire</t>
+  </si>
+  <si>
+    <t>Trees outside forests partially disturbed in the current interval without signif. height increase after with fire</t>
+  </si>
+  <si>
+    <t>Trees outside forests partially disturbed in the current interval without signif. height increase after without fire</t>
+  </si>
+  <si>
+    <t>Oil palm not disturbed in the current interval with fire</t>
+  </si>
+  <si>
+    <t>Oil palm not disturbed in the current interval without fire</t>
+  </si>
+  <si>
+    <t>Planted trees not disturbed in the current interval with fire</t>
+  </si>
+  <si>
+    <t>Planted trees not disturbed in the current interval without fire</t>
+  </si>
+  <si>
+    <t>Young secondary natural forest with fire</t>
+  </si>
+  <si>
+    <t>Young secondary natural forest without fire</t>
+  </si>
+  <si>
+    <t>Primary forest undisturbed since model start with fire</t>
+  </si>
+  <si>
+    <t>Primary forest undisturbed since model start without fire</t>
+  </si>
+  <si>
+    <t>Old secondary forest undisturbed since model start with fire</t>
+  </si>
+  <si>
+    <t>Old secondary forest undisturbed since model start without fire</t>
+  </si>
+  <si>
+    <t>Trees outside forests not disturbed in the current interval with fire</t>
+  </si>
+  <si>
+    <t>Trees outside forests not disturbed in the current interval without fire</t>
+  </si>
+  <si>
+    <t>Annual cropland converted to short vegetation with fire</t>
+  </si>
+  <si>
+    <t>Annual cropland converted to short vegetation without fire</t>
+  </si>
+  <si>
+    <t>Annual cropland converted to water</t>
+  </si>
+  <si>
+    <t>Annual cropland converted to anything else with fire</t>
+  </si>
+  <si>
+    <t>Annual cropland converted to anything else without fire</t>
+  </si>
+  <si>
+    <t>Cropland remaining cropland with fire</t>
+  </si>
+  <si>
+    <t>Cropland remaining cropland without fire</t>
+  </si>
+  <si>
+    <t>Short vegetation gain</t>
+  </si>
+  <si>
+    <t>Short vegetation loss converted to water</t>
+  </si>
+  <si>
+    <t>Short vegetation loss converted to non-water with fire</t>
+  </si>
+  <si>
+    <t>Short vegetation loss converted to non-water without fire</t>
+  </si>
+  <si>
+    <t>Short vegetation remaining short vegetation with fire</t>
+  </si>
+  <si>
+    <t>Short vegetation remaining short vegetation without fire</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -291,6 +532,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FF8C8C8C"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -313,9 +561,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -597,13 +848,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C76"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>76</v>
       </c>
@@ -614,7 +865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3">
       <c r="A2">
         <v>1110000</v>
       </c>
@@ -626,7 +877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3">
       <c r="A3">
         <v>1120000</v>
       </c>
@@ -638,7 +889,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3">
       <c r="A4">
         <v>1210000</v>
       </c>
@@ -650,7 +901,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3">
       <c r="A5">
         <v>1220000</v>
       </c>
@@ -662,7 +913,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3">
       <c r="A6">
         <v>2000000</v>
       </c>
@@ -674,7 +925,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3">
       <c r="A7">
         <v>2111000</v>
       </c>
@@ -686,7 +937,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3">
       <c r="A8">
         <v>2112000</v>
       </c>
@@ -698,7 +949,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3">
       <c r="A9">
         <v>2121100</v>
       </c>
@@ -710,7 +961,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3">
       <c r="A10">
         <v>2121200</v>
       </c>
@@ -722,7 +973,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3">
       <c r="A11">
         <v>2122100</v>
       </c>
@@ -734,7 +985,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3">
       <c r="A12">
         <v>2122200</v>
       </c>
@@ -746,7 +997,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3">
       <c r="A13">
         <v>2123100</v>
       </c>
@@ -758,7 +1009,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3">
       <c r="A14">
         <v>2123200</v>
       </c>
@@ -770,7 +1021,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3">
       <c r="A15">
         <v>2124100</v>
       </c>
@@ -782,7 +1033,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3">
       <c r="A16">
         <v>2124200</v>
       </c>
@@ -794,7 +1045,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3">
       <c r="A17">
         <v>2125100</v>
       </c>
@@ -806,7 +1057,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3">
       <c r="A18">
         <v>2125200</v>
       </c>
@@ -818,7 +1069,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3">
       <c r="A19">
         <v>2211100</v>
       </c>
@@ -830,7 +1081,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3">
       <c r="A20">
         <v>2211200</v>
       </c>
@@ -842,7 +1093,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3">
       <c r="A21">
         <v>2212110</v>
       </c>
@@ -854,7 +1105,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3">
       <c r="A22">
         <v>2212120</v>
       </c>
@@ -866,7 +1117,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3">
       <c r="A23">
         <v>2212210</v>
       </c>
@@ -878,7 +1129,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3">
       <c r="A24">
         <v>2212220</v>
       </c>
@@ -890,7 +1141,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3">
       <c r="A25">
         <v>2213110</v>
       </c>
@@ -902,7 +1153,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3">
       <c r="A26">
         <v>2213120</v>
       </c>
@@ -914,7 +1165,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3">
       <c r="A27">
         <v>2213210</v>
       </c>
@@ -926,7 +1177,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3">
       <c r="A28">
         <v>2213220</v>
       </c>
@@ -938,7 +1189,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3">
       <c r="A29">
         <v>2214100</v>
       </c>
@@ -950,7 +1201,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3">
       <c r="A30">
         <v>2214200</v>
       </c>
@@ -962,7 +1213,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3">
       <c r="A31">
         <v>2215100</v>
       </c>
@@ -974,7 +1225,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3">
       <c r="A32">
         <v>2215200</v>
       </c>
@@ -986,7 +1237,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3">
       <c r="A33">
         <v>2221100</v>
       </c>
@@ -998,7 +1249,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3">
       <c r="A34">
         <v>2221200</v>
       </c>
@@ -1010,7 +1261,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3">
       <c r="A35">
         <v>2222100</v>
       </c>
@@ -1022,7 +1273,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3">
       <c r="A36">
         <v>2222200</v>
       </c>
@@ -1034,7 +1285,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3">
       <c r="A37">
         <v>2223100</v>
       </c>
@@ -1046,7 +1297,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3">
       <c r="A38">
         <v>2223200</v>
       </c>
@@ -1058,7 +1309,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3">
       <c r="A39">
         <v>3110000</v>
       </c>
@@ -1070,7 +1321,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3">
       <c r="A40">
         <v>3120000</v>
       </c>
@@ -1082,7 +1333,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3">
       <c r="A41">
         <v>3211111</v>
       </c>
@@ -1094,7 +1345,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3">
       <c r="A42">
         <v>3211112</v>
       </c>
@@ -1106,7 +1357,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3">
       <c r="A43">
         <v>3211121</v>
       </c>
@@ -1118,7 +1369,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3">
       <c r="A44">
         <v>3211122</v>
       </c>
@@ -1130,7 +1381,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3">
       <c r="A45">
         <v>3211211</v>
       </c>
@@ -1142,7 +1393,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3">
       <c r="A46">
         <v>3211212</v>
       </c>
@@ -1154,7 +1405,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3">
       <c r="A47">
         <v>3211221</v>
       </c>
@@ -1166,7 +1417,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3">
       <c r="A48">
         <v>3211222</v>
       </c>
@@ -1178,7 +1429,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3">
       <c r="A49">
         <v>3212111</v>
       </c>
@@ -1190,7 +1441,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3">
       <c r="A50">
         <v>3212112</v>
       </c>
@@ -1202,7 +1453,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3">
       <c r="A51">
         <v>3212121</v>
       </c>
@@ -1214,7 +1465,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3">
       <c r="A52">
         <v>3212122</v>
       </c>
@@ -1226,7 +1477,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3">
       <c r="A53">
         <v>3212211</v>
       </c>
@@ -1238,7 +1489,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3">
       <c r="A54">
         <v>3212212</v>
       </c>
@@ -1250,7 +1501,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3">
       <c r="A55">
         <v>3212221</v>
       </c>
@@ -1262,7 +1513,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3">
       <c r="A56">
         <v>3212222</v>
       </c>
@@ -1274,7 +1525,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3">
       <c r="A57">
         <v>3221110</v>
       </c>
@@ -1286,7 +1537,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3">
       <c r="A58">
         <v>3221120</v>
       </c>
@@ -1298,7 +1549,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3">
       <c r="A59">
         <v>3221210</v>
       </c>
@@ -1310,7 +1561,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3">
       <c r="A60">
         <v>3221220</v>
       </c>
@@ -1322,7 +1573,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3">
       <c r="A61">
         <v>3222111</v>
       </c>
@@ -1334,7 +1585,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3">
       <c r="A62">
         <v>3222112</v>
       </c>
@@ -1346,7 +1597,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3">
       <c r="A63">
         <v>3222121</v>
       </c>
@@ -1358,7 +1609,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3">
       <c r="A64">
         <v>3222122</v>
       </c>
@@ -1370,7 +1621,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3">
       <c r="A65">
         <v>3222210</v>
       </c>
@@ -1382,7 +1633,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:3">
       <c r="A66">
         <v>3222220</v>
       </c>
@@ -1394,7 +1645,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3">
       <c r="A67">
         <v>4100000</v>
       </c>
@@ -1406,7 +1657,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3">
       <c r="A68">
         <v>4210000</v>
       </c>
@@ -1418,7 +1669,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3">
       <c r="A69">
         <v>4220000</v>
       </c>
@@ -1430,7 +1681,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3">
       <c r="A70">
         <v>4310000</v>
       </c>
@@ -1442,7 +1693,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3">
       <c r="A71">
         <v>4320000</v>
       </c>
@@ -1454,7 +1705,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3">
       <c r="A72">
         <v>5100000</v>
       </c>
@@ -1466,7 +1717,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:3">
       <c r="A73">
         <v>5210000</v>
       </c>
@@ -1478,7 +1729,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3">
       <c r="A74">
         <v>5220000</v>
       </c>
@@ -1490,7 +1741,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3">
       <c r="A75">
         <v>5310000</v>
       </c>
@@ -1502,7 +1753,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3">
       <c r="A76">
         <v>5320000</v>
       </c>
@@ -1517,4 +1768,1314 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{853D7656-B308-4E3A-9467-98AD8F1F4D68}">
+  <dimension ref="A1:D81"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.26953125" customWidth="1"/>
+    <col min="3" max="3" width="22.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2">
+        <v>211</v>
+      </c>
+      <c r="B2" t="str">
+        <f>A2&amp;REPT("0",8-LEN(A2))</f>
+        <v>21100000</v>
+      </c>
+      <c r="C2" t="str">
+        <f>_xlfn.CONCAT("n",B2)</f>
+        <v>n21100000</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="2">
+        <v>212</v>
+      </c>
+      <c r="B3" t="str">
+        <f t="shared" ref="B3:B62" si="0">A3&amp;REPT("0",8-LEN(A3))</f>
+        <v>21200000</v>
+      </c>
+      <c r="C3" t="str">
+        <f t="shared" ref="C3:C62" si="1">_xlfn.CONCAT("n",B3)</f>
+        <v>n21200000</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="2">
+        <v>221</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>22100000</v>
+      </c>
+      <c r="C4" t="str">
+        <f t="shared" si="1"/>
+        <v>n22100000</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="2">
+        <v>222</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>22200000</v>
+      </c>
+      <c r="C5" t="str">
+        <f t="shared" si="1"/>
+        <v>n22200000</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="2">
+        <v>3119</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>31190000</v>
+      </c>
+      <c r="C6" t="str">
+        <f t="shared" si="1"/>
+        <v>n31190000</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="2">
+        <v>3112</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>31120000</v>
+      </c>
+      <c r="C7" t="str">
+        <f t="shared" si="1"/>
+        <v>n31120000</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="2">
+        <v>312119</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>31211900</v>
+      </c>
+      <c r="C8" t="str">
+        <f t="shared" si="1"/>
+        <v>n31211900</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="2">
+        <v>312112</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>31211200</v>
+      </c>
+      <c r="C9" t="str">
+        <f t="shared" si="1"/>
+        <v>n31211200</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="2">
+        <v>312129</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>31212900</v>
+      </c>
+      <c r="C10" t="str">
+        <f t="shared" si="1"/>
+        <v>n31212900</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="2">
+        <v>312122</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>31212200</v>
+      </c>
+      <c r="C11" t="str">
+        <f t="shared" si="1"/>
+        <v>n31212200</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="2">
+        <v>312219</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>31221900</v>
+      </c>
+      <c r="C12" t="str">
+        <f t="shared" si="1"/>
+        <v>n31221900</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="2">
+        <v>312212</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>31221200</v>
+      </c>
+      <c r="C13" t="str">
+        <f t="shared" si="1"/>
+        <v>n31221200</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="2">
+        <v>312229</v>
+      </c>
+      <c r="B14" t="str">
+        <f t="shared" si="0"/>
+        <v>31222900</v>
+      </c>
+      <c r="C14" t="str">
+        <f t="shared" si="1"/>
+        <v>n31222900</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="2">
+        <v>312222</v>
+      </c>
+      <c r="B15" t="str">
+        <f t="shared" si="0"/>
+        <v>31222200</v>
+      </c>
+      <c r="C15" t="str">
+        <f t="shared" si="1"/>
+        <v>n31222200</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="2">
+        <v>312319</v>
+      </c>
+      <c r="B16" t="str">
+        <f t="shared" si="0"/>
+        <v>31231900</v>
+      </c>
+      <c r="C16" t="str">
+        <f t="shared" si="1"/>
+        <v>n31231900</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="2">
+        <v>312312</v>
+      </c>
+      <c r="B17" t="str">
+        <f t="shared" si="0"/>
+        <v>31231200</v>
+      </c>
+      <c r="C17" t="str">
+        <f t="shared" si="1"/>
+        <v>n31231200</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="2">
+        <v>312329</v>
+      </c>
+      <c r="B18" t="str">
+        <f t="shared" si="0"/>
+        <v>31232900</v>
+      </c>
+      <c r="C18" t="str">
+        <f t="shared" si="1"/>
+        <v>n31232900</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="2">
+        <v>312322</v>
+      </c>
+      <c r="B19" t="str">
+        <f t="shared" si="0"/>
+        <v>31232200</v>
+      </c>
+      <c r="C19" t="str">
+        <f t="shared" si="1"/>
+        <v>n31232200</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="2">
+        <v>312412</v>
+      </c>
+      <c r="B20" t="str">
+        <f t="shared" si="0"/>
+        <v>31241200</v>
+      </c>
+      <c r="C20" t="str">
+        <f t="shared" si="1"/>
+        <v>n31241200</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="2">
+        <v>312422</v>
+      </c>
+      <c r="B21" t="str">
+        <f t="shared" si="0"/>
+        <v>31242200</v>
+      </c>
+      <c r="C21" t="str">
+        <f t="shared" si="1"/>
+        <v>n31242200</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="2">
+        <v>32119</v>
+      </c>
+      <c r="B22" t="str">
+        <f t="shared" si="0"/>
+        <v>32119000</v>
+      </c>
+      <c r="C22" t="str">
+        <f t="shared" si="1"/>
+        <v>n32119000</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="2">
+        <v>32112</v>
+      </c>
+      <c r="B23" t="str">
+        <f t="shared" si="0"/>
+        <v>32112000</v>
+      </c>
+      <c r="C23" t="str">
+        <f t="shared" si="1"/>
+        <v>n32112000</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="2">
+        <v>321219</v>
+      </c>
+      <c r="B24" t="str">
+        <f t="shared" si="0"/>
+        <v>32121900</v>
+      </c>
+      <c r="C24" t="str">
+        <f t="shared" si="1"/>
+        <v>n32121900</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="2">
+        <v>321212</v>
+      </c>
+      <c r="B25" t="str">
+        <f t="shared" si="0"/>
+        <v>32121200</v>
+      </c>
+      <c r="C25" t="str">
+        <f t="shared" si="1"/>
+        <v>n32121200</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="2">
+        <v>321229</v>
+      </c>
+      <c r="B26" t="str">
+        <f t="shared" si="0"/>
+        <v>32122900</v>
+      </c>
+      <c r="C26" t="str">
+        <f t="shared" si="1"/>
+        <v>n32122900</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="2">
+        <v>321222</v>
+      </c>
+      <c r="B27" t="str">
+        <f t="shared" si="0"/>
+        <v>32122200</v>
+      </c>
+      <c r="C27" t="str">
+        <f t="shared" si="1"/>
+        <v>n32122200</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="2">
+        <v>32139</v>
+      </c>
+      <c r="B28" t="str">
+        <f t="shared" si="0"/>
+        <v>32139000</v>
+      </c>
+      <c r="C28" t="str">
+        <f t="shared" si="1"/>
+        <v>n32139000</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="2">
+        <v>32132</v>
+      </c>
+      <c r="B29" t="str">
+        <f t="shared" si="0"/>
+        <v>32132000</v>
+      </c>
+      <c r="C29" t="str">
+        <f t="shared" si="1"/>
+        <v>n32132000</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="2">
+        <v>32142</v>
+      </c>
+      <c r="B30" t="str">
+        <f t="shared" si="0"/>
+        <v>32142000</v>
+      </c>
+      <c r="C30" t="str">
+        <f t="shared" si="1"/>
+        <v>n32142000</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="2">
+        <v>32219</v>
+      </c>
+      <c r="B31" t="str">
+        <f t="shared" si="0"/>
+        <v>32219000</v>
+      </c>
+      <c r="C31" t="str">
+        <f t="shared" si="1"/>
+        <v>n32219000</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="2">
+        <v>32212</v>
+      </c>
+      <c r="B32" t="str">
+        <f t="shared" si="0"/>
+        <v>32212000</v>
+      </c>
+      <c r="C32" t="str">
+        <f t="shared" si="1"/>
+        <v>n32212000</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="2">
+        <v>32229</v>
+      </c>
+      <c r="B33" t="str">
+        <f t="shared" si="0"/>
+        <v>32229000</v>
+      </c>
+      <c r="C33" t="str">
+        <f t="shared" si="1"/>
+        <v>n32229000</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="2">
+        <v>32222</v>
+      </c>
+      <c r="B34" t="str">
+        <f t="shared" si="0"/>
+        <v>32222000</v>
+      </c>
+      <c r="C34" t="str">
+        <f t="shared" si="1"/>
+        <v>n32222000</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" s="2">
+        <v>32239</v>
+      </c>
+      <c r="B35" t="str">
+        <f t="shared" si="0"/>
+        <v>32239000</v>
+      </c>
+      <c r="C35" t="str">
+        <f t="shared" si="1"/>
+        <v>n32239000</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="2">
+        <v>32232</v>
+      </c>
+      <c r="B36" t="str">
+        <f t="shared" si="0"/>
+        <v>32232000</v>
+      </c>
+      <c r="C36" t="str">
+        <f t="shared" si="1"/>
+        <v>n32232000</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" s="2">
+        <v>32242</v>
+      </c>
+      <c r="B37" t="str">
+        <f t="shared" si="0"/>
+        <v>32242000</v>
+      </c>
+      <c r="C37" t="str">
+        <f t="shared" si="1"/>
+        <v>n32242000</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" s="2">
+        <v>419</v>
+      </c>
+      <c r="B38" t="str">
+        <f t="shared" si="0"/>
+        <v>41900000</v>
+      </c>
+      <c r="C38" t="str">
+        <f t="shared" si="1"/>
+        <v>n41900000</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="2">
+        <v>412</v>
+      </c>
+      <c r="B39" t="str">
+        <f t="shared" si="0"/>
+        <v>41200000</v>
+      </c>
+      <c r="C39" t="str">
+        <f t="shared" si="1"/>
+        <v>n41200000</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="2">
+        <v>4211119</v>
+      </c>
+      <c r="B40" t="str">
+        <f t="shared" si="0"/>
+        <v>42111190</v>
+      </c>
+      <c r="C40" t="str">
+        <f t="shared" si="1"/>
+        <v>n42111190</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="2">
+        <v>4211112</v>
+      </c>
+      <c r="B41" t="str">
+        <f t="shared" si="0"/>
+        <v>42111120</v>
+      </c>
+      <c r="C41" t="str">
+        <f t="shared" si="1"/>
+        <v>n42111120</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" s="2">
+        <v>4211129</v>
+      </c>
+      <c r="B42" t="str">
+        <f t="shared" si="0"/>
+        <v>42111290</v>
+      </c>
+      <c r="C42" t="str">
+        <f t="shared" si="1"/>
+        <v>n42111290</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="2">
+        <v>4211122</v>
+      </c>
+      <c r="B43" t="str">
+        <f t="shared" si="0"/>
+        <v>42111220</v>
+      </c>
+      <c r="C43" t="str">
+        <f t="shared" si="1"/>
+        <v>n42111220</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" s="2">
+        <v>4211219</v>
+      </c>
+      <c r="B44" t="str">
+        <f t="shared" si="0"/>
+        <v>42112190</v>
+      </c>
+      <c r="C44" t="str">
+        <f t="shared" si="1"/>
+        <v>n42112190</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" s="2">
+        <v>4211212</v>
+      </c>
+      <c r="B45" t="str">
+        <f t="shared" si="0"/>
+        <v>42112120</v>
+      </c>
+      <c r="C45" t="str">
+        <f t="shared" si="1"/>
+        <v>n42112120</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="2">
+        <v>4211229</v>
+      </c>
+      <c r="B46" t="str">
+        <f t="shared" si="0"/>
+        <v>42112290</v>
+      </c>
+      <c r="C46" t="str">
+        <f t="shared" si="1"/>
+        <v>n42112290</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="2">
+        <v>4211222</v>
+      </c>
+      <c r="B47" t="str">
+        <f t="shared" si="0"/>
+        <v>42112220</v>
+      </c>
+      <c r="C47" t="str">
+        <f t="shared" si="1"/>
+        <v>n42112220</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" s="2">
+        <v>4212119</v>
+      </c>
+      <c r="B48" t="str">
+        <f t="shared" si="0"/>
+        <v>42121190</v>
+      </c>
+      <c r="C48" t="str">
+        <f t="shared" si="1"/>
+        <v>n42121190</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" s="2">
+        <v>4212112</v>
+      </c>
+      <c r="B49" t="str">
+        <f t="shared" si="0"/>
+        <v>42121120</v>
+      </c>
+      <c r="C49" t="str">
+        <f t="shared" si="1"/>
+        <v>n42121120</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" s="2">
+        <v>4212129</v>
+      </c>
+      <c r="B50" t="str">
+        <f t="shared" si="0"/>
+        <v>42121290</v>
+      </c>
+      <c r="C50" t="str">
+        <f t="shared" si="1"/>
+        <v>n42121290</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" s="2">
+        <v>4212122</v>
+      </c>
+      <c r="B51" t="str">
+        <f t="shared" si="0"/>
+        <v>42121220</v>
+      </c>
+      <c r="C51" t="str">
+        <f t="shared" si="1"/>
+        <v>n42121220</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52" s="2">
+        <v>4212219</v>
+      </c>
+      <c r="B52" t="str">
+        <f t="shared" si="0"/>
+        <v>42122190</v>
+      </c>
+      <c r="C52" t="str">
+        <f t="shared" si="1"/>
+        <v>n42122190</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" s="2">
+        <v>4212212</v>
+      </c>
+      <c r="B53" t="str">
+        <f t="shared" si="0"/>
+        <v>42122120</v>
+      </c>
+      <c r="C53" t="str">
+        <f t="shared" si="1"/>
+        <v>n42122120</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" s="2">
+        <v>4212229</v>
+      </c>
+      <c r="B54" t="str">
+        <f t="shared" si="0"/>
+        <v>42122290</v>
+      </c>
+      <c r="C54" t="str">
+        <f t="shared" si="1"/>
+        <v>n42122290</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55" s="2">
+        <v>4212222</v>
+      </c>
+      <c r="B55" t="str">
+        <f t="shared" si="0"/>
+        <v>42122220</v>
+      </c>
+      <c r="C55" t="str">
+        <f t="shared" si="1"/>
+        <v>n42122220</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" s="2">
+        <v>422119</v>
+      </c>
+      <c r="B56" t="str">
+        <f t="shared" si="0"/>
+        <v>42211900</v>
+      </c>
+      <c r="C56" t="str">
+        <f t="shared" si="1"/>
+        <v>n42211900</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" s="2">
+        <v>422112</v>
+      </c>
+      <c r="B57" t="str">
+        <f t="shared" si="0"/>
+        <v>42211200</v>
+      </c>
+      <c r="C57" t="str">
+        <f t="shared" si="1"/>
+        <v>n42211200</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" s="2">
+        <v>422129</v>
+      </c>
+      <c r="B58" t="str">
+        <f t="shared" si="0"/>
+        <v>42212900</v>
+      </c>
+      <c r="C58" t="str">
+        <f t="shared" si="1"/>
+        <v>n42212900</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" s="2">
+        <v>422122</v>
+      </c>
+      <c r="B59" t="str">
+        <f t="shared" si="0"/>
+        <v>42212200</v>
+      </c>
+      <c r="C59" t="str">
+        <f t="shared" si="1"/>
+        <v>n42212200</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" s="2">
+        <v>4222119</v>
+      </c>
+      <c r="B60" t="str">
+        <f t="shared" si="0"/>
+        <v>42221190</v>
+      </c>
+      <c r="C60" t="str">
+        <f t="shared" si="1"/>
+        <v>n42221190</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" s="2">
+        <v>4222112</v>
+      </c>
+      <c r="B61" t="str">
+        <f t="shared" si="0"/>
+        <v>42221120</v>
+      </c>
+      <c r="C61" t="str">
+        <f t="shared" si="1"/>
+        <v>n42221120</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="2">
+        <v>42221219</v>
+      </c>
+      <c r="B62" t="str">
+        <f t="shared" si="0"/>
+        <v>42221219</v>
+      </c>
+      <c r="C62" t="str">
+        <f t="shared" si="1"/>
+        <v>n42221219</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" s="2">
+        <v>42221212</v>
+      </c>
+      <c r="B63" t="str">
+        <f t="shared" ref="B63:B81" si="2">A63&amp;REPT("0",8-LEN(A63))</f>
+        <v>42221212</v>
+      </c>
+      <c r="C63" t="str">
+        <f t="shared" ref="C63:C81" si="3">_xlfn.CONCAT("n",B63)</f>
+        <v>n42221212</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="A64" s="2">
+        <v>42221229</v>
+      </c>
+      <c r="B64" t="str">
+        <f t="shared" si="2"/>
+        <v>42221229</v>
+      </c>
+      <c r="C64" t="str">
+        <f t="shared" si="3"/>
+        <v>n42221229</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" s="2">
+        <v>42221222</v>
+      </c>
+      <c r="B65" t="str">
+        <f t="shared" si="2"/>
+        <v>42221222</v>
+      </c>
+      <c r="C65" t="str">
+        <f t="shared" si="3"/>
+        <v>n42221222</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="2">
+        <v>422229</v>
+      </c>
+      <c r="B66" t="str">
+        <f t="shared" si="2"/>
+        <v>42222900</v>
+      </c>
+      <c r="C66" t="str">
+        <f t="shared" si="3"/>
+        <v>n42222900</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" s="2">
+        <v>422222</v>
+      </c>
+      <c r="B67" t="str">
+        <f t="shared" si="2"/>
+        <v>42222200</v>
+      </c>
+      <c r="C67" t="str">
+        <f t="shared" si="3"/>
+        <v>n42222200</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4">
+      <c r="A68" s="2">
+        <v>51</v>
+      </c>
+      <c r="B68" t="str">
+        <f t="shared" si="2"/>
+        <v>51000000</v>
+      </c>
+      <c r="C68" t="str">
+        <f t="shared" si="3"/>
+        <v>n51000000</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
+      <c r="A69" s="2">
+        <v>5219</v>
+      </c>
+      <c r="B69" t="str">
+        <f t="shared" si="2"/>
+        <v>52190000</v>
+      </c>
+      <c r="C69" t="str">
+        <f t="shared" si="3"/>
+        <v>n52190000</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" s="2">
+        <v>5212</v>
+      </c>
+      <c r="B70" t="str">
+        <f t="shared" si="2"/>
+        <v>52120000</v>
+      </c>
+      <c r="C70" t="str">
+        <f t="shared" si="3"/>
+        <v>n52120000</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71" s="2">
+        <v>5222</v>
+      </c>
+      <c r="B71" t="str">
+        <f t="shared" si="2"/>
+        <v>52220000</v>
+      </c>
+      <c r="C71" t="str">
+        <f t="shared" si="3"/>
+        <v>n52220000</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72" s="2">
+        <v>5239</v>
+      </c>
+      <c r="B72" t="str">
+        <f t="shared" si="2"/>
+        <v>52390000</v>
+      </c>
+      <c r="C72" t="str">
+        <f t="shared" si="3"/>
+        <v>n52390000</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4">
+      <c r="A73" s="2">
+        <v>5232</v>
+      </c>
+      <c r="B73" t="str">
+        <f t="shared" si="2"/>
+        <v>52320000</v>
+      </c>
+      <c r="C73" t="str">
+        <f t="shared" si="3"/>
+        <v>n52320000</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4">
+      <c r="A74" s="2">
+        <v>539</v>
+      </c>
+      <c r="B74" t="str">
+        <f t="shared" si="2"/>
+        <v>53900000</v>
+      </c>
+      <c r="C74" t="str">
+        <f t="shared" si="3"/>
+        <v>n53900000</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4">
+      <c r="A75" s="2">
+        <v>532</v>
+      </c>
+      <c r="B75" t="str">
+        <f t="shared" si="2"/>
+        <v>53200000</v>
+      </c>
+      <c r="C75" t="str">
+        <f t="shared" si="3"/>
+        <v>n53200000</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4">
+      <c r="A76" s="2">
+        <v>61</v>
+      </c>
+      <c r="B76" t="str">
+        <f t="shared" si="2"/>
+        <v>61000000</v>
+      </c>
+      <c r="C76" t="str">
+        <f t="shared" si="3"/>
+        <v>n61000000</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4">
+      <c r="A77" s="2">
+        <v>6212</v>
+      </c>
+      <c r="B77" t="str">
+        <f t="shared" si="2"/>
+        <v>62120000</v>
+      </c>
+      <c r="C77" t="str">
+        <f t="shared" si="3"/>
+        <v>n62120000</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4">
+      <c r="A78" s="2">
+        <v>6229</v>
+      </c>
+      <c r="B78" t="str">
+        <f t="shared" si="2"/>
+        <v>62290000</v>
+      </c>
+      <c r="C78" t="str">
+        <f t="shared" si="3"/>
+        <v>n62290000</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4">
+      <c r="A79" s="2">
+        <v>6222</v>
+      </c>
+      <c r="B79" t="str">
+        <f t="shared" si="2"/>
+        <v>62220000</v>
+      </c>
+      <c r="C79" t="str">
+        <f t="shared" si="3"/>
+        <v>n62220000</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4">
+      <c r="A80" s="2">
+        <v>639</v>
+      </c>
+      <c r="B80" t="str">
+        <f t="shared" si="2"/>
+        <v>63900000</v>
+      </c>
+      <c r="C80" t="str">
+        <f t="shared" si="3"/>
+        <v>n63900000</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4">
+      <c r="A81" s="2">
+        <v>632</v>
+      </c>
+      <c r="B81" t="str">
+        <f t="shared" si="2"/>
+        <v>63200000</v>
+      </c>
+      <c r="C81" t="str">
+        <f t="shared" si="3"/>
+        <v>n63200000</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Although I'm still aggregating the 1884-chunk outputs for v0.4.0, I am going to merge this branch so I can move to 0.4.2 (2000-2024).
</commit_message>
<xml_diff>
--- a/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
+++ b/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIS\git\AFOLU_GHG_flux_model\src\LULUCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EEA2BDC-D595-4D86-A8F5-322A3E5634B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0F9CF9F-790C-420A-9E70-7FFD995A4E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-9180" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1795,7 +1795,7 @@
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2">
+      <c r="A2" s="2">
         <v>211</v>
       </c>
       <c r="B2" t="str">

</xml_diff>

<commit_message>
Ran core model and post-processing for Cerrado. Working on zonal stats in notebook now.
</commit_message>
<xml_diff>
--- a/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
+++ b/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIS\git\AFOLU_GHG_flux_model\src\LULUCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0F9CF9F-790C-420A-9E70-7FFD995A4E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F00498-839A-4870-BF33-17CBAC702092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-9180" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16515" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="v030_20250430" sheetId="1" r:id="rId1"/>
     <sheet name="v040_20250805" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">v040_20250805!$A$1:$F$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -37,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="173">
   <si>
     <t>meaning</t>
   </si>
@@ -511,6 +514,51 @@
   </si>
   <si>
     <t>Short vegetation remaining short vegetation without fire</t>
+  </si>
+  <si>
+    <t>broad_class</t>
+  </si>
+  <si>
+    <t>detailed_class</t>
+  </si>
+  <si>
+    <t>tree_gain</t>
+  </si>
+  <si>
+    <t>tree_loss</t>
+  </si>
+  <si>
+    <t>crop_gain</t>
+  </si>
+  <si>
+    <t>crop_loss</t>
+  </si>
+  <si>
+    <t>tree_tree_undisturbed</t>
+  </si>
+  <si>
+    <t>tree_tree_disturbed</t>
+  </si>
+  <si>
+    <t>crop_crop_undisturbed</t>
+  </si>
+  <si>
+    <t>short_veg_gain</t>
+  </si>
+  <si>
+    <t>short_veg_loss</t>
+  </si>
+  <si>
+    <t>short_veg_short_veg_undisturbed</t>
+  </si>
+  <si>
+    <t>tree</t>
+  </si>
+  <si>
+    <t>crop</t>
+  </si>
+  <si>
+    <t>short_veg</t>
   </si>
 </sst>
 </file>
@@ -549,7 +597,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -557,16 +605,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1772,15 +1834,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{853D7656-B308-4E3A-9467-98AD8F1F4D68}">
-  <dimension ref="A1:D81"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.26953125" customWidth="1"/>
-    <col min="3" max="3" width="22.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="132.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>78</v>
       </c>
@@ -1793,8 +1858,14 @@
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" s="2">
         <v>211</v>
       </c>
@@ -1809,8 +1880,14 @@
       <c r="D2" s="2" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="E2" t="s">
+        <v>170</v>
+      </c>
+      <c r="F2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" s="2">
         <v>212</v>
       </c>
@@ -1825,8 +1902,14 @@
       <c r="D3" s="2" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="E3" t="s">
+        <v>170</v>
+      </c>
+      <c r="F3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" s="2">
         <v>221</v>
       </c>
@@ -1841,24 +1924,36 @@
       <c r="D4" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="2">
+      <c r="E4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="4" customFormat="1">
+      <c r="A5" s="3">
         <v>222</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B5" s="4" t="str">
         <f t="shared" si="0"/>
         <v>22200000</v>
       </c>
-      <c r="C5" t="str">
+      <c r="C5" s="4" t="str">
         <f t="shared" si="1"/>
         <v>n22200000</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="E5" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" s="2">
         <v>3119</v>
       </c>
@@ -1873,8 +1968,14 @@
       <c r="D6" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="E6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" s="2">
         <v>3112</v>
       </c>
@@ -1889,8 +1990,14 @@
       <c r="D7" s="2" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="8" spans="1:4">
+      <c r="E7" t="s">
+        <v>170</v>
+      </c>
+      <c r="F7" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" s="2">
         <v>312119</v>
       </c>
@@ -1905,8 +2012,14 @@
       <c r="D8" s="2" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="E8" t="s">
+        <v>170</v>
+      </c>
+      <c r="F8" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" s="2">
         <v>312112</v>
       </c>
@@ -1921,8 +2034,14 @@
       <c r="D9" s="2" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
+      <c r="E9" t="s">
+        <v>170</v>
+      </c>
+      <c r="F9" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" s="2">
         <v>312129</v>
       </c>
@@ -1937,8 +2056,14 @@
       <c r="D10" s="2" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="11" spans="1:4">
+      <c r="E10" t="s">
+        <v>170</v>
+      </c>
+      <c r="F10" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" s="2">
         <v>312122</v>
       </c>
@@ -1953,8 +2078,14 @@
       <c r="D11" s="2" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="12" spans="1:4">
+      <c r="E11" t="s">
+        <v>170</v>
+      </c>
+      <c r="F11" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" s="2">
         <v>312219</v>
       </c>
@@ -1969,8 +2100,14 @@
       <c r="D12" s="2" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="13" spans="1:4">
+      <c r="E12" t="s">
+        <v>170</v>
+      </c>
+      <c r="F12" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" s="2">
         <v>312212</v>
       </c>
@@ -1985,8 +2122,14 @@
       <c r="D13" s="2" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
+      <c r="E13" t="s">
+        <v>170</v>
+      </c>
+      <c r="F13" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" s="2">
         <v>312229</v>
       </c>
@@ -2001,8 +2144,14 @@
       <c r="D14" s="2" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="15" spans="1:4">
+      <c r="E14" t="s">
+        <v>170</v>
+      </c>
+      <c r="F14" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15" s="2">
         <v>312222</v>
       </c>
@@ -2017,8 +2166,14 @@
       <c r="D15" s="2" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
+      <c r="E15" t="s">
+        <v>170</v>
+      </c>
+      <c r="F15" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" s="2">
         <v>312319</v>
       </c>
@@ -2033,8 +2188,14 @@
       <c r="D16" s="2" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="E16" t="s">
+        <v>170</v>
+      </c>
+      <c r="F16" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
       <c r="A17" s="2">
         <v>312312</v>
       </c>
@@ -2049,8 +2210,14 @@
       <c r="D17" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
+      <c r="E17" t="s">
+        <v>170</v>
+      </c>
+      <c r="F17" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18" s="2">
         <v>312329</v>
       </c>
@@ -2065,8 +2232,14 @@
       <c r="D18" s="2" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
+      <c r="E18" t="s">
+        <v>170</v>
+      </c>
+      <c r="F18" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19" s="2">
         <v>312322</v>
       </c>
@@ -2081,8 +2254,14 @@
       <c r="D19" s="2" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="20" spans="1:4">
+      <c r="E19" t="s">
+        <v>170</v>
+      </c>
+      <c r="F19" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20" s="2">
         <v>312412</v>
       </c>
@@ -2097,8 +2276,14 @@
       <c r="D20" s="2" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="21" spans="1:4">
+      <c r="E20" t="s">
+        <v>170</v>
+      </c>
+      <c r="F20" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="A21" s="2">
         <v>312422</v>
       </c>
@@ -2113,8 +2298,14 @@
       <c r="D21" s="2" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="22" spans="1:4">
+      <c r="E21" t="s">
+        <v>170</v>
+      </c>
+      <c r="F21" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
       <c r="A22" s="2">
         <v>32119</v>
       </c>
@@ -2129,8 +2320,14 @@
       <c r="D22" s="2" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
+      <c r="E22" t="s">
+        <v>170</v>
+      </c>
+      <c r="F22" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
       <c r="A23" s="2">
         <v>32112</v>
       </c>
@@ -2145,8 +2342,14 @@
       <c r="D23" s="2" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="24" spans="1:4">
+      <c r="E23" t="s">
+        <v>170</v>
+      </c>
+      <c r="F23" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
       <c r="A24" s="2">
         <v>321219</v>
       </c>
@@ -2161,8 +2364,14 @@
       <c r="D24" s="2" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="25" spans="1:4">
+      <c r="E24" t="s">
+        <v>170</v>
+      </c>
+      <c r="F24" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
       <c r="A25" s="2">
         <v>321212</v>
       </c>
@@ -2177,8 +2386,14 @@
       <c r="D25" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="26" spans="1:4">
+      <c r="E25" t="s">
+        <v>170</v>
+      </c>
+      <c r="F25" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
       <c r="A26" s="2">
         <v>321229</v>
       </c>
@@ -2193,8 +2408,14 @@
       <c r="D26" s="2" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="27" spans="1:4">
+      <c r="E26" t="s">
+        <v>170</v>
+      </c>
+      <c r="F26" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
       <c r="A27" s="2">
         <v>321222</v>
       </c>
@@ -2209,8 +2430,14 @@
       <c r="D27" s="2" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="28" spans="1:4">
+      <c r="E27" t="s">
+        <v>170</v>
+      </c>
+      <c r="F27" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
       <c r="A28" s="2">
         <v>32139</v>
       </c>
@@ -2225,8 +2452,14 @@
       <c r="D28" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="29" spans="1:4">
+      <c r="E28" t="s">
+        <v>170</v>
+      </c>
+      <c r="F28" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
       <c r="A29" s="2">
         <v>32132</v>
       </c>
@@ -2241,8 +2474,14 @@
       <c r="D29" s="2" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="30" spans="1:4">
+      <c r="E29" t="s">
+        <v>170</v>
+      </c>
+      <c r="F29" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
       <c r="A30" s="2">
         <v>32142</v>
       </c>
@@ -2257,8 +2496,14 @@
       <c r="D30" s="2" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="31" spans="1:4">
+      <c r="E30" t="s">
+        <v>170</v>
+      </c>
+      <c r="F30" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
       <c r="A31" s="2">
         <v>32219</v>
       </c>
@@ -2273,8 +2518,14 @@
       <c r="D31" s="2" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="32" spans="1:4">
+      <c r="E31" t="s">
+        <v>170</v>
+      </c>
+      <c r="F31" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
       <c r="A32" s="2">
         <v>32212</v>
       </c>
@@ -2289,8 +2540,14 @@
       <c r="D32" s="2" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="33" spans="1:4">
+      <c r="E32" t="s">
+        <v>170</v>
+      </c>
+      <c r="F32" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
       <c r="A33" s="2">
         <v>32229</v>
       </c>
@@ -2305,8 +2562,14 @@
       <c r="D33" s="2" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="34" spans="1:4">
+      <c r="E33" t="s">
+        <v>170</v>
+      </c>
+      <c r="F33" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
       <c r="A34" s="2">
         <v>32222</v>
       </c>
@@ -2321,8 +2584,14 @@
       <c r="D34" s="2" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="35" spans="1:4">
+      <c r="E34" t="s">
+        <v>170</v>
+      </c>
+      <c r="F34" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
       <c r="A35" s="2">
         <v>32239</v>
       </c>
@@ -2337,8 +2606,14 @@
       <c r="D35" s="2" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="36" spans="1:4">
+      <c r="E35" t="s">
+        <v>170</v>
+      </c>
+      <c r="F35" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
       <c r="A36" s="2">
         <v>32232</v>
       </c>
@@ -2353,24 +2628,36 @@
       <c r="D36" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="37" spans="1:4">
-      <c r="A37" s="2">
+      <c r="E36" t="s">
+        <v>170</v>
+      </c>
+      <c r="F36" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" s="4" customFormat="1">
+      <c r="A37" s="3">
         <v>32242</v>
       </c>
-      <c r="B37" t="str">
+      <c r="B37" s="4" t="str">
         <f t="shared" si="0"/>
         <v>32242000</v>
       </c>
-      <c r="C37" t="str">
+      <c r="C37" s="4" t="str">
         <f t="shared" si="1"/>
         <v>n32242000</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="D37" s="3" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="38" spans="1:4">
+      <c r="E37" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
       <c r="A38" s="2">
         <v>419</v>
       </c>
@@ -2385,8 +2672,14 @@
       <c r="D38" s="2" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="39" spans="1:4">
+      <c r="E38" t="s">
+        <v>170</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
       <c r="A39" s="2">
         <v>412</v>
       </c>
@@ -2401,8 +2694,14 @@
       <c r="D39" s="2" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="40" spans="1:4">
+      <c r="E39" t="s">
+        <v>170</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
       <c r="A40" s="2">
         <v>4211119</v>
       </c>
@@ -2417,8 +2716,14 @@
       <c r="D40" s="2" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="41" spans="1:4">
+      <c r="E40" t="s">
+        <v>170</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
       <c r="A41" s="2">
         <v>4211112</v>
       </c>
@@ -2433,8 +2738,14 @@
       <c r="D41" s="2" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="42" spans="1:4">
+      <c r="E41" t="s">
+        <v>170</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
       <c r="A42" s="2">
         <v>4211129</v>
       </c>
@@ -2449,8 +2760,14 @@
       <c r="D42" s="2" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="43" spans="1:4">
+      <c r="E42" t="s">
+        <v>170</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
       <c r="A43" s="2">
         <v>4211122</v>
       </c>
@@ -2465,8 +2782,14 @@
       <c r="D43" s="2" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="44" spans="1:4">
+      <c r="E43" t="s">
+        <v>170</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
       <c r="A44" s="2">
         <v>4211219</v>
       </c>
@@ -2481,8 +2804,14 @@
       <c r="D44" s="2" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="45" spans="1:4">
+      <c r="E44" t="s">
+        <v>170</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
       <c r="A45" s="2">
         <v>4211212</v>
       </c>
@@ -2497,8 +2826,14 @@
       <c r="D45" s="2" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="46" spans="1:4">
+      <c r="E45" t="s">
+        <v>170</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
       <c r="A46" s="2">
         <v>4211229</v>
       </c>
@@ -2513,8 +2848,14 @@
       <c r="D46" s="2" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="47" spans="1:4">
+      <c r="E46" t="s">
+        <v>170</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
       <c r="A47" s="2">
         <v>4211222</v>
       </c>
@@ -2529,8 +2870,14 @@
       <c r="D47" s="2" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="48" spans="1:4">
+      <c r="E47" t="s">
+        <v>170</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
       <c r="A48" s="2">
         <v>4212119</v>
       </c>
@@ -2545,8 +2892,14 @@
       <c r="D48" s="2" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="49" spans="1:4">
+      <c r="E48" t="s">
+        <v>170</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
       <c r="A49" s="2">
         <v>4212112</v>
       </c>
@@ -2561,8 +2914,14 @@
       <c r="D49" s="2" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="50" spans="1:4">
+      <c r="E49" t="s">
+        <v>170</v>
+      </c>
+      <c r="F49" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
       <c r="A50" s="2">
         <v>4212129</v>
       </c>
@@ -2577,8 +2936,14 @@
       <c r="D50" s="2" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="51" spans="1:4">
+      <c r="E50" t="s">
+        <v>170</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
       <c r="A51" s="2">
         <v>4212122</v>
       </c>
@@ -2593,8 +2958,14 @@
       <c r="D51" s="2" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="52" spans="1:4">
+      <c r="E51" t="s">
+        <v>170</v>
+      </c>
+      <c r="F51" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
       <c r="A52" s="2">
         <v>4212219</v>
       </c>
@@ -2609,8 +2980,14 @@
       <c r="D52" s="2" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="53" spans="1:4">
+      <c r="E52" t="s">
+        <v>170</v>
+      </c>
+      <c r="F52" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
       <c r="A53" s="2">
         <v>4212212</v>
       </c>
@@ -2625,8 +3002,14 @@
       <c r="D53" s="2" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="54" spans="1:4">
+      <c r="E53" t="s">
+        <v>170</v>
+      </c>
+      <c r="F53" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
       <c r="A54" s="2">
         <v>4212229</v>
       </c>
@@ -2641,8 +3024,14 @@
       <c r="D54" s="2" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="55" spans="1:4">
+      <c r="E54" t="s">
+        <v>170</v>
+      </c>
+      <c r="F54" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
       <c r="A55" s="2">
         <v>4212222</v>
       </c>
@@ -2657,8 +3046,14 @@
       <c r="D55" s="2" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="56" spans="1:4">
+      <c r="E55" t="s">
+        <v>170</v>
+      </c>
+      <c r="F55" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
       <c r="A56" s="2">
         <v>422119</v>
       </c>
@@ -2673,8 +3068,14 @@
       <c r="D56" s="2" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="57" spans="1:4">
+      <c r="E56" t="s">
+        <v>170</v>
+      </c>
+      <c r="F56" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
       <c r="A57" s="2">
         <v>422112</v>
       </c>
@@ -2689,8 +3090,14 @@
       <c r="D57" s="2" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="58" spans="1:4">
+      <c r="E57" t="s">
+        <v>170</v>
+      </c>
+      <c r="F57" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
       <c r="A58" s="2">
         <v>422129</v>
       </c>
@@ -2705,8 +3112,14 @@
       <c r="D58" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="59" spans="1:4">
+      <c r="E58" t="s">
+        <v>170</v>
+      </c>
+      <c r="F58" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
       <c r="A59" s="2">
         <v>422122</v>
       </c>
@@ -2721,8 +3134,14 @@
       <c r="D59" s="2" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="60" spans="1:4">
+      <c r="E59" t="s">
+        <v>170</v>
+      </c>
+      <c r="F59" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
       <c r="A60" s="2">
         <v>4222119</v>
       </c>
@@ -2737,8 +3156,14 @@
       <c r="D60" s="2" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="61" spans="1:4">
+      <c r="E60" t="s">
+        <v>170</v>
+      </c>
+      <c r="F60" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
       <c r="A61" s="2">
         <v>4222112</v>
       </c>
@@ -2753,8 +3178,14 @@
       <c r="D61" s="2" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="62" spans="1:4">
+      <c r="E61" t="s">
+        <v>170</v>
+      </c>
+      <c r="F61" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
       <c r="A62" s="2">
         <v>42221219</v>
       </c>
@@ -2769,8 +3200,14 @@
       <c r="D62" s="2" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="63" spans="1:4">
+      <c r="E62" t="s">
+        <v>170</v>
+      </c>
+      <c r="F62" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
       <c r="A63" s="2">
         <v>42221212</v>
       </c>
@@ -2785,8 +3222,14 @@
       <c r="D63" s="2" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="64" spans="1:4">
+      <c r="E63" t="s">
+        <v>170</v>
+      </c>
+      <c r="F63" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
       <c r="A64" s="2">
         <v>42221229</v>
       </c>
@@ -2801,8 +3244,14 @@
       <c r="D64" s="2" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="65" spans="1:4">
+      <c r="E64" t="s">
+        <v>170</v>
+      </c>
+      <c r="F64" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
       <c r="A65" s="2">
         <v>42221222</v>
       </c>
@@ -2817,8 +3266,14 @@
       <c r="D65" s="2" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="66" spans="1:4">
+      <c r="E65" t="s">
+        <v>170</v>
+      </c>
+      <c r="F65" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
       <c r="A66" s="2">
         <v>422229</v>
       </c>
@@ -2833,24 +3288,36 @@
       <c r="D66" s="2" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="67" spans="1:4">
-      <c r="A67" s="2">
+      <c r="E66" t="s">
+        <v>170</v>
+      </c>
+      <c r="F66" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" s="4" customFormat="1">
+      <c r="A67" s="3">
         <v>422222</v>
       </c>
-      <c r="B67" t="str">
+      <c r="B67" s="4" t="str">
         <f t="shared" si="2"/>
         <v>42222200</v>
       </c>
-      <c r="C67" t="str">
+      <c r="C67" s="4" t="str">
         <f t="shared" si="3"/>
         <v>n42222200</v>
       </c>
-      <c r="D67" s="2" t="s">
+      <c r="D67" s="3" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="68" spans="1:4">
+      <c r="E67" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
       <c r="A68" s="2">
         <v>51</v>
       </c>
@@ -2865,8 +3332,14 @@
       <c r="D68" s="2" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="69" spans="1:4">
+      <c r="E68" t="s">
+        <v>171</v>
+      </c>
+      <c r="F68" s="5" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
       <c r="A69" s="2">
         <v>5219</v>
       </c>
@@ -2881,8 +3354,14 @@
       <c r="D69" s="2" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="70" spans="1:4">
+      <c r="E69" t="s">
+        <v>171</v>
+      </c>
+      <c r="F69" s="5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
       <c r="A70" s="2">
         <v>5212</v>
       </c>
@@ -2897,8 +3376,14 @@
       <c r="D70" s="2" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="71" spans="1:4">
+      <c r="E70" t="s">
+        <v>171</v>
+      </c>
+      <c r="F70" s="5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
       <c r="A71" s="2">
         <v>5222</v>
       </c>
@@ -2913,8 +3398,14 @@
       <c r="D71" s="2" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="72" spans="1:4">
+      <c r="E71" t="s">
+        <v>171</v>
+      </c>
+      <c r="F71" s="5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
       <c r="A72" s="2">
         <v>5239</v>
       </c>
@@ -2929,8 +3420,14 @@
       <c r="D72" s="2" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="73" spans="1:4">
+      <c r="E72" t="s">
+        <v>171</v>
+      </c>
+      <c r="F72" s="5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
       <c r="A73" s="2">
         <v>5232</v>
       </c>
@@ -2945,8 +3442,14 @@
       <c r="D73" s="2" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="74" spans="1:4">
+      <c r="E73" t="s">
+        <v>171</v>
+      </c>
+      <c r="F73" s="5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6">
       <c r="A74" s="2">
         <v>539</v>
       </c>
@@ -2961,24 +3464,36 @@
       <c r="D74" s="2" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="75" spans="1:4">
-      <c r="A75" s="2">
+      <c r="E74" t="s">
+        <v>171</v>
+      </c>
+      <c r="F74" s="5" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" s="4" customFormat="1">
+      <c r="A75" s="3">
         <v>532</v>
       </c>
-      <c r="B75" t="str">
+      <c r="B75" s="4" t="str">
         <f t="shared" si="2"/>
         <v>53200000</v>
       </c>
-      <c r="C75" t="str">
+      <c r="C75" s="4" t="str">
         <f t="shared" si="3"/>
         <v>n53200000</v>
       </c>
-      <c r="D75" s="2" t="s">
+      <c r="D75" s="3" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="76" spans="1:4">
+      <c r="E75" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6">
       <c r="A76" s="2">
         <v>61</v>
       </c>
@@ -2993,8 +3508,14 @@
       <c r="D76" s="2" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="77" spans="1:4">
+      <c r="E76" t="s">
+        <v>172</v>
+      </c>
+      <c r="F76" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6">
       <c r="A77" s="2">
         <v>6212</v>
       </c>
@@ -3009,8 +3530,14 @@
       <c r="D77" s="2" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="78" spans="1:4">
+      <c r="E77" t="s">
+        <v>172</v>
+      </c>
+      <c r="F77" s="5" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6">
       <c r="A78" s="2">
         <v>6229</v>
       </c>
@@ -3025,8 +3552,14 @@
       <c r="D78" s="2" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="79" spans="1:4">
+      <c r="E78" t="s">
+        <v>172</v>
+      </c>
+      <c r="F78" s="5" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6">
       <c r="A79" s="2">
         <v>6222</v>
       </c>
@@ -3041,8 +3574,14 @@
       <c r="D79" s="2" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="80" spans="1:4">
+      <c r="E79" t="s">
+        <v>172</v>
+      </c>
+      <c r="F79" s="5" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6">
       <c r="A80" s="2">
         <v>639</v>
       </c>
@@ -3057,24 +3596,37 @@
       <c r="D80" s="2" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="81" spans="1:4">
-      <c r="A81" s="2">
+      <c r="E80" t="s">
+        <v>172</v>
+      </c>
+      <c r="F80" s="5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" s="4" customFormat="1">
+      <c r="A81" s="3">
         <v>632</v>
       </c>
-      <c r="B81" t="str">
+      <c r="B81" s="4" t="str">
         <f t="shared" si="2"/>
         <v>63200000</v>
       </c>
-      <c r="C81" t="str">
+      <c r="C81" s="4" t="str">
         <f t="shared" si="3"/>
         <v>n63200000</v>
       </c>
-      <c r="D81" s="2" t="s">
+      <c r="D81" s="3" t="s">
         <v>157</v>
       </c>
+      <c r="E81" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>169</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F1" xr:uid="{853D7656-B308-4E3A-9467-98AD8F1F4D68}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Cerrado zonal stats notebook working now. Checked emissions in 2005, net flux in 2010, and removals in 2024 against ArcPro zonal statistics as table. All three pairs match.
</commit_message>
<xml_diff>
--- a/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
+++ b/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIS\git\AFOLU_GHG_flux_model\src\LULUCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F00498-839A-4870-BF33-17CBAC702092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8699F0B-351A-4CEA-80F5-1A723F17F819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16515" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-9180" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="v030_20250430" sheetId="1" r:id="rId1"/>
-    <sheet name="v040_20250805" sheetId="2" r:id="rId2"/>
+    <sheet name="v042_20250805" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">v040_20250805!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">v042_20250805!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="175">
   <si>
     <t>meaning</t>
   </si>
@@ -559,6 +559,12 @@
   </si>
   <si>
     <t>short_veg</t>
+  </si>
+  <si>
+    <t>Not in decision tree</t>
+  </si>
+  <si>
+    <t>None</t>
   </si>
 </sst>
 </file>
@@ -618,7 +624,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -628,6 +634,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1834,7 +1843,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{853D7656-B308-4E3A-9467-98AD8F1F4D68}">
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
@@ -1971,7 +1980,7 @@
       <c r="E6" t="s">
         <v>170</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" t="s">
         <v>161</v>
       </c>
     </row>
@@ -2675,7 +2684,7 @@
       <c r="E38" t="s">
         <v>170</v>
       </c>
-      <c r="F38" s="5" t="s">
+      <c r="F38" t="s">
         <v>161</v>
       </c>
     </row>
@@ -2697,7 +2706,7 @@
       <c r="E39" t="s">
         <v>170</v>
       </c>
-      <c r="F39" s="5" t="s">
+      <c r="F39" t="s">
         <v>161</v>
       </c>
     </row>
@@ -2719,7 +2728,7 @@
       <c r="E40" t="s">
         <v>170</v>
       </c>
-      <c r="F40" s="5" t="s">
+      <c r="F40" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2741,7 +2750,7 @@
       <c r="E41" t="s">
         <v>170</v>
       </c>
-      <c r="F41" s="5" t="s">
+      <c r="F41" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2763,7 +2772,7 @@
       <c r="E42" t="s">
         <v>170</v>
       </c>
-      <c r="F42" s="5" t="s">
+      <c r="F42" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2785,7 +2794,7 @@
       <c r="E43" t="s">
         <v>170</v>
       </c>
-      <c r="F43" s="5" t="s">
+      <c r="F43" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2807,7 +2816,7 @@
       <c r="E44" t="s">
         <v>170</v>
       </c>
-      <c r="F44" s="5" t="s">
+      <c r="F44" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2829,7 +2838,7 @@
       <c r="E45" t="s">
         <v>170</v>
       </c>
-      <c r="F45" s="5" t="s">
+      <c r="F45" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2851,7 +2860,7 @@
       <c r="E46" t="s">
         <v>170</v>
       </c>
-      <c r="F46" s="5" t="s">
+      <c r="F46" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2873,7 +2882,7 @@
       <c r="E47" t="s">
         <v>170</v>
       </c>
-      <c r="F47" s="5" t="s">
+      <c r="F47" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2895,7 +2904,7 @@
       <c r="E48" t="s">
         <v>170</v>
       </c>
-      <c r="F48" s="5" t="s">
+      <c r="F48" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2917,7 +2926,7 @@
       <c r="E49" t="s">
         <v>170</v>
       </c>
-      <c r="F49" s="5" t="s">
+      <c r="F49" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2939,7 +2948,7 @@
       <c r="E50" t="s">
         <v>170</v>
       </c>
-      <c r="F50" s="5" t="s">
+      <c r="F50" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2961,7 +2970,7 @@
       <c r="E51" t="s">
         <v>170</v>
       </c>
-      <c r="F51" s="5" t="s">
+      <c r="F51" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2983,7 +2992,7 @@
       <c r="E52" t="s">
         <v>170</v>
       </c>
-      <c r="F52" s="5" t="s">
+      <c r="F52" t="s">
         <v>165</v>
       </c>
     </row>
@@ -3005,7 +3014,7 @@
       <c r="E53" t="s">
         <v>170</v>
       </c>
-      <c r="F53" s="5" t="s">
+      <c r="F53" t="s">
         <v>165</v>
       </c>
     </row>
@@ -3027,7 +3036,7 @@
       <c r="E54" t="s">
         <v>170</v>
       </c>
-      <c r="F54" s="5" t="s">
+      <c r="F54" t="s">
         <v>165</v>
       </c>
     </row>
@@ -3049,7 +3058,7 @@
       <c r="E55" t="s">
         <v>170</v>
       </c>
-      <c r="F55" s="5" t="s">
+      <c r="F55" t="s">
         <v>165</v>
       </c>
     </row>
@@ -3071,7 +3080,7 @@
       <c r="E56" t="s">
         <v>170</v>
       </c>
-      <c r="F56" s="5" t="s">
+      <c r="F56" t="s">
         <v>164</v>
       </c>
     </row>
@@ -3212,11 +3221,11 @@
         <v>42221212</v>
       </c>
       <c r="B63" t="str">
-        <f t="shared" ref="B63:B81" si="2">A63&amp;REPT("0",8-LEN(A63))</f>
+        <f t="shared" ref="B63:B82" si="2">A63&amp;REPT("0",8-LEN(A63))</f>
         <v>42221212</v>
       </c>
       <c r="C63" t="str">
-        <f t="shared" ref="C63:C81" si="3">_xlfn.CONCAT("n",B63)</f>
+        <f t="shared" ref="C63:C82" si="3">_xlfn.CONCAT("n",B63)</f>
         <v>n42221212</v>
       </c>
       <c r="D63" s="2" t="s">
@@ -3335,7 +3344,7 @@
       <c r="E68" t="s">
         <v>171</v>
       </c>
-      <c r="F68" s="5" t="s">
+      <c r="F68" t="s">
         <v>162</v>
       </c>
     </row>
@@ -3357,7 +3366,7 @@
       <c r="E69" t="s">
         <v>171</v>
       </c>
-      <c r="F69" s="5" t="s">
+      <c r="F69" t="s">
         <v>163</v>
       </c>
     </row>
@@ -3379,7 +3388,7 @@
       <c r="E70" t="s">
         <v>171</v>
       </c>
-      <c r="F70" s="5" t="s">
+      <c r="F70" t="s">
         <v>163</v>
       </c>
     </row>
@@ -3401,7 +3410,7 @@
       <c r="E71" t="s">
         <v>171</v>
       </c>
-      <c r="F71" s="5" t="s">
+      <c r="F71" t="s">
         <v>163</v>
       </c>
     </row>
@@ -3423,7 +3432,7 @@
       <c r="E72" t="s">
         <v>171</v>
       </c>
-      <c r="F72" s="5" t="s">
+      <c r="F72" t="s">
         <v>163</v>
       </c>
     </row>
@@ -3445,7 +3454,7 @@
       <c r="E73" t="s">
         <v>171</v>
       </c>
-      <c r="F73" s="5" t="s">
+      <c r="F73" t="s">
         <v>163</v>
       </c>
     </row>
@@ -3467,7 +3476,7 @@
       <c r="E74" t="s">
         <v>171</v>
       </c>
-      <c r="F74" s="5" t="s">
+      <c r="F74" t="s">
         <v>166</v>
       </c>
     </row>
@@ -3511,7 +3520,7 @@
       <c r="E76" t="s">
         <v>172</v>
       </c>
-      <c r="F76" s="5" t="s">
+      <c r="F76" t="s">
         <v>167</v>
       </c>
     </row>
@@ -3533,7 +3542,7 @@
       <c r="E77" t="s">
         <v>172</v>
       </c>
-      <c r="F77" s="5" t="s">
+      <c r="F77" t="s">
         <v>168</v>
       </c>
     </row>
@@ -3555,7 +3564,7 @@
       <c r="E78" t="s">
         <v>172</v>
       </c>
-      <c r="F78" s="5" t="s">
+      <c r="F78" t="s">
         <v>168</v>
       </c>
     </row>
@@ -3577,7 +3586,7 @@
       <c r="E79" t="s">
         <v>172</v>
       </c>
-      <c r="F79" s="5" t="s">
+      <c r="F79" t="s">
         <v>168</v>
       </c>
     </row>
@@ -3599,7 +3608,7 @@
       <c r="E80" t="s">
         <v>172</v>
       </c>
-      <c r="F80" s="5" t="s">
+      <c r="F80" t="s">
         <v>169</v>
       </c>
     </row>
@@ -3623,6 +3632,28 @@
       </c>
       <c r="F81" s="4" t="s">
         <v>169</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6">
+      <c r="A82" s="5">
+        <v>7</v>
+      </c>
+      <c r="B82" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>70000000</v>
+      </c>
+      <c r="C82" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n70000000</v>
+      </c>
+      <c r="D82" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="E82" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="F82" s="6" t="s">
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tested different configurations for running zonal stats on Cerrado LULUCF outputs. A different notebook for each.
</commit_message>
<xml_diff>
--- a/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
+++ b/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIS\git\AFOLU_GHG_flux_model\src\LULUCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8699F0B-351A-4CEA-80F5-1A723F17F819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0524C3B-2A53-42E1-A53B-4DCB6B01D89A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-9180" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -564,7 +564,7 @@
     <t>Not in decision tree</t>
   </si>
   <si>
-    <t>None</t>
+    <t>no_flux</t>
   </si>
 </sst>
 </file>
@@ -624,7 +624,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -634,10 +634,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3635,24 +3631,24 @@
       </c>
     </row>
     <row r="82" spans="1:6">
-      <c r="A82" s="5">
+      <c r="A82" s="2">
         <v>7</v>
       </c>
-      <c r="B82" s="6" t="str">
+      <c r="B82" t="str">
         <f t="shared" si="2"/>
         <v>70000000</v>
       </c>
-      <c r="C82" s="6" t="str">
+      <c r="C82" t="str">
         <f t="shared" si="3"/>
         <v>n70000000</v>
       </c>
-      <c r="D82" s="5" t="s">
+      <c r="D82" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="E82" s="6" t="s">
+      <c r="E82" t="s">
         <v>174</v>
       </c>
-      <c r="F82" s="6" t="s">
+      <c r="F82" t="s">
         <v>174</v>
       </c>
     </row>

</xml_diff>

<commit_message>
SOC timeseries script works for 1x1 and 10x10 deg density and change geotif creation. Units are correct now. Going to include masking by OGH organic soil extent now.
</commit_message>
<xml_diff>
--- a/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
+++ b/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
@@ -8,18 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIS\git\AFOLU_GHG_flux_model\src\LULUCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0524C3B-2A53-42E1-A53B-4DCB6B01D89A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E38FF9-D75E-4C6D-A6A6-5997748DFEA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-9180" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="v030_20250430" sheetId="1" r:id="rId1"/>
-    <sheet name="v042_20250805" sheetId="2" r:id="rId2"/>
+    <sheet name="v040_20250713" sheetId="3" r:id="rId2"/>
+    <sheet name="v042_20250805" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">v042_20250805!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">v040_20250713!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">v042_20250805!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="175">
   <si>
     <t>meaning</t>
   </si>
@@ -1838,6 +1841,1828 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{190A0781-4690-4C4E-8E78-7EC47B65C964}">
+  <dimension ref="A1:F82"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="132.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="2">
+        <v>211</v>
+      </c>
+      <c r="B2" t="str">
+        <f>A2&amp;REPT("0",8-LEN(A2))</f>
+        <v>21100000</v>
+      </c>
+      <c r="C2" t="str">
+        <f>_xlfn.CONCAT("n",B2)</f>
+        <v>n21100000</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E2" t="s">
+        <v>170</v>
+      </c>
+      <c r="F2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="2">
+        <v>212</v>
+      </c>
+      <c r="B3" t="str">
+        <f t="shared" ref="B3:B66" si="0">A3&amp;REPT("0",8-LEN(A3))</f>
+        <v>21200000</v>
+      </c>
+      <c r="C3" t="str">
+        <f t="shared" ref="C3:C66" si="1">_xlfn.CONCAT("n",B3)</f>
+        <v>n21200000</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E3" t="s">
+        <v>170</v>
+      </c>
+      <c r="F3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="2">
+        <v>221</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>22100000</v>
+      </c>
+      <c r="C4" t="str">
+        <f t="shared" si="1"/>
+        <v>n22100000</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="4" customFormat="1">
+      <c r="A5" s="3">
+        <v>222</v>
+      </c>
+      <c r="B5" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>22200000</v>
+      </c>
+      <c r="C5" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>n22200000</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="2">
+        <v>3119</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>31190000</v>
+      </c>
+      <c r="C6" t="str">
+        <f t="shared" si="1"/>
+        <v>n31190000</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="2">
+        <v>3112</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>31120000</v>
+      </c>
+      <c r="C7" t="str">
+        <f t="shared" si="1"/>
+        <v>n31120000</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E7" t="s">
+        <v>170</v>
+      </c>
+      <c r="F7" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="2">
+        <v>312119</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>31211900</v>
+      </c>
+      <c r="C8" t="str">
+        <f t="shared" si="1"/>
+        <v>n31211900</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E8" t="s">
+        <v>170</v>
+      </c>
+      <c r="F8" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="2">
+        <v>312112</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>31211200</v>
+      </c>
+      <c r="C9" t="str">
+        <f t="shared" si="1"/>
+        <v>n31211200</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E9" t="s">
+        <v>170</v>
+      </c>
+      <c r="F9" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="2">
+        <v>312129</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>31212900</v>
+      </c>
+      <c r="C10" t="str">
+        <f t="shared" si="1"/>
+        <v>n31212900</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10" t="s">
+        <v>170</v>
+      </c>
+      <c r="F10" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="2">
+        <v>312122</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>31212200</v>
+      </c>
+      <c r="C11" t="str">
+        <f t="shared" si="1"/>
+        <v>n31212200</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E11" t="s">
+        <v>170</v>
+      </c>
+      <c r="F11" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="2">
+        <v>312219</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>31221900</v>
+      </c>
+      <c r="C12" t="str">
+        <f t="shared" si="1"/>
+        <v>n31221900</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E12" t="s">
+        <v>170</v>
+      </c>
+      <c r="F12" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="2">
+        <v>312212</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>31221200</v>
+      </c>
+      <c r="C13" t="str">
+        <f t="shared" si="1"/>
+        <v>n31221200</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E13" t="s">
+        <v>170</v>
+      </c>
+      <c r="F13" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="2">
+        <v>312229</v>
+      </c>
+      <c r="B14" t="str">
+        <f t="shared" si="0"/>
+        <v>31222900</v>
+      </c>
+      <c r="C14" t="str">
+        <f t="shared" si="1"/>
+        <v>n31222900</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E14" t="s">
+        <v>170</v>
+      </c>
+      <c r="F14" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="2">
+        <v>312222</v>
+      </c>
+      <c r="B15" t="str">
+        <f t="shared" si="0"/>
+        <v>31222200</v>
+      </c>
+      <c r="C15" t="str">
+        <f t="shared" si="1"/>
+        <v>n31222200</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E15" t="s">
+        <v>170</v>
+      </c>
+      <c r="F15" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="2">
+        <v>312319</v>
+      </c>
+      <c r="B16" t="str">
+        <f t="shared" si="0"/>
+        <v>31231900</v>
+      </c>
+      <c r="C16" t="str">
+        <f t="shared" si="1"/>
+        <v>n31231900</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E16" t="s">
+        <v>170</v>
+      </c>
+      <c r="F16" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="2">
+        <v>312312</v>
+      </c>
+      <c r="B17" t="str">
+        <f t="shared" si="0"/>
+        <v>31231200</v>
+      </c>
+      <c r="C17" t="str">
+        <f t="shared" si="1"/>
+        <v>n31231200</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E17" t="s">
+        <v>170</v>
+      </c>
+      <c r="F17" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="2">
+        <v>312329</v>
+      </c>
+      <c r="B18" t="str">
+        <f t="shared" si="0"/>
+        <v>31232900</v>
+      </c>
+      <c r="C18" t="str">
+        <f t="shared" si="1"/>
+        <v>n31232900</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E18" t="s">
+        <v>170</v>
+      </c>
+      <c r="F18" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="2">
+        <v>312322</v>
+      </c>
+      <c r="B19" t="str">
+        <f t="shared" si="0"/>
+        <v>31232200</v>
+      </c>
+      <c r="C19" t="str">
+        <f t="shared" si="1"/>
+        <v>n31232200</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E19" t="s">
+        <v>170</v>
+      </c>
+      <c r="F19" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="2">
+        <v>312412</v>
+      </c>
+      <c r="B20" t="str">
+        <f t="shared" si="0"/>
+        <v>31241200</v>
+      </c>
+      <c r="C20" t="str">
+        <f t="shared" si="1"/>
+        <v>n31241200</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E20" t="s">
+        <v>170</v>
+      </c>
+      <c r="F20" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="2">
+        <v>312422</v>
+      </c>
+      <c r="B21" t="str">
+        <f t="shared" si="0"/>
+        <v>31242200</v>
+      </c>
+      <c r="C21" t="str">
+        <f t="shared" si="1"/>
+        <v>n31242200</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E21" t="s">
+        <v>170</v>
+      </c>
+      <c r="F21" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="2">
+        <v>32119</v>
+      </c>
+      <c r="B22" t="str">
+        <f t="shared" si="0"/>
+        <v>32119000</v>
+      </c>
+      <c r="C22" t="str">
+        <f t="shared" si="1"/>
+        <v>n32119000</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E22" t="s">
+        <v>170</v>
+      </c>
+      <c r="F22" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="2">
+        <v>32112</v>
+      </c>
+      <c r="B23" t="str">
+        <f t="shared" si="0"/>
+        <v>32112000</v>
+      </c>
+      <c r="C23" t="str">
+        <f t="shared" si="1"/>
+        <v>n32112000</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E23" t="s">
+        <v>170</v>
+      </c>
+      <c r="F23" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="2">
+        <v>321219</v>
+      </c>
+      <c r="B24" t="str">
+        <f t="shared" si="0"/>
+        <v>32121900</v>
+      </c>
+      <c r="C24" t="str">
+        <f t="shared" si="1"/>
+        <v>n32121900</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E24" t="s">
+        <v>170</v>
+      </c>
+      <c r="F24" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" s="2">
+        <v>321212</v>
+      </c>
+      <c r="B25" t="str">
+        <f t="shared" si="0"/>
+        <v>32121200</v>
+      </c>
+      <c r="C25" t="str">
+        <f t="shared" si="1"/>
+        <v>n32121200</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E25" t="s">
+        <v>170</v>
+      </c>
+      <c r="F25" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" s="2">
+        <v>321229</v>
+      </c>
+      <c r="B26" t="str">
+        <f t="shared" si="0"/>
+        <v>32122900</v>
+      </c>
+      <c r="C26" t="str">
+        <f t="shared" si="1"/>
+        <v>n32122900</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E26" t="s">
+        <v>170</v>
+      </c>
+      <c r="F26" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" s="2">
+        <v>321222</v>
+      </c>
+      <c r="B27" t="str">
+        <f t="shared" si="0"/>
+        <v>32122200</v>
+      </c>
+      <c r="C27" t="str">
+        <f t="shared" si="1"/>
+        <v>n32122200</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E27" t="s">
+        <v>170</v>
+      </c>
+      <c r="F27" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="2">
+        <v>32139</v>
+      </c>
+      <c r="B28" t="str">
+        <f t="shared" si="0"/>
+        <v>32139000</v>
+      </c>
+      <c r="C28" t="str">
+        <f t="shared" si="1"/>
+        <v>n32139000</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E28" t="s">
+        <v>170</v>
+      </c>
+      <c r="F28" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" s="2">
+        <v>32132</v>
+      </c>
+      <c r="B29" t="str">
+        <f t="shared" si="0"/>
+        <v>32132000</v>
+      </c>
+      <c r="C29" t="str">
+        <f t="shared" si="1"/>
+        <v>n32132000</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E29" t="s">
+        <v>170</v>
+      </c>
+      <c r="F29" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="2">
+        <v>32142</v>
+      </c>
+      <c r="B30" t="str">
+        <f t="shared" si="0"/>
+        <v>32142000</v>
+      </c>
+      <c r="C30" t="str">
+        <f t="shared" si="1"/>
+        <v>n32142000</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E30" t="s">
+        <v>170</v>
+      </c>
+      <c r="F30" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" s="2">
+        <v>32219</v>
+      </c>
+      <c r="B31" t="str">
+        <f t="shared" si="0"/>
+        <v>32219000</v>
+      </c>
+      <c r="C31" t="str">
+        <f t="shared" si="1"/>
+        <v>n32219000</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E31" t="s">
+        <v>170</v>
+      </c>
+      <c r="F31" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" s="2">
+        <v>32212</v>
+      </c>
+      <c r="B32" t="str">
+        <f t="shared" si="0"/>
+        <v>32212000</v>
+      </c>
+      <c r="C32" t="str">
+        <f t="shared" si="1"/>
+        <v>n32212000</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E32" t="s">
+        <v>170</v>
+      </c>
+      <c r="F32" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" s="2">
+        <v>32229</v>
+      </c>
+      <c r="B33" t="str">
+        <f t="shared" si="0"/>
+        <v>32229000</v>
+      </c>
+      <c r="C33" t="str">
+        <f t="shared" si="1"/>
+        <v>n32229000</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E33" t="s">
+        <v>170</v>
+      </c>
+      <c r="F33" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" s="2">
+        <v>32222</v>
+      </c>
+      <c r="B34" t="str">
+        <f t="shared" si="0"/>
+        <v>32222000</v>
+      </c>
+      <c r="C34" t="str">
+        <f t="shared" si="1"/>
+        <v>n32222000</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E34" t="s">
+        <v>170</v>
+      </c>
+      <c r="F34" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="2">
+        <v>32239</v>
+      </c>
+      <c r="B35" t="str">
+        <f t="shared" si="0"/>
+        <v>32239000</v>
+      </c>
+      <c r="C35" t="str">
+        <f t="shared" si="1"/>
+        <v>n32239000</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E35" t="s">
+        <v>170</v>
+      </c>
+      <c r="F35" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" s="2">
+        <v>32232</v>
+      </c>
+      <c r="B36" t="str">
+        <f t="shared" si="0"/>
+        <v>32232000</v>
+      </c>
+      <c r="C36" t="str">
+        <f t="shared" si="1"/>
+        <v>n32232000</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E36" t="s">
+        <v>170</v>
+      </c>
+      <c r="F36" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" s="4" customFormat="1">
+      <c r="A37" s="3">
+        <v>32242</v>
+      </c>
+      <c r="B37" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>32242000</v>
+      </c>
+      <c r="C37" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>n32242000</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" s="2">
+        <v>419</v>
+      </c>
+      <c r="B38" t="str">
+        <f t="shared" si="0"/>
+        <v>41900000</v>
+      </c>
+      <c r="C38" t="str">
+        <f t="shared" si="1"/>
+        <v>n41900000</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E38" t="s">
+        <v>170</v>
+      </c>
+      <c r="F38" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="2">
+        <v>412</v>
+      </c>
+      <c r="B39" t="str">
+        <f t="shared" si="0"/>
+        <v>41200000</v>
+      </c>
+      <c r="C39" t="str">
+        <f t="shared" si="1"/>
+        <v>n41200000</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E39" t="s">
+        <v>170</v>
+      </c>
+      <c r="F39" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="2">
+        <v>4211119</v>
+      </c>
+      <c r="B40" t="str">
+        <f t="shared" si="0"/>
+        <v>42111190</v>
+      </c>
+      <c r="C40" t="str">
+        <f t="shared" si="1"/>
+        <v>n42111190</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E40" t="s">
+        <v>170</v>
+      </c>
+      <c r="F40" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" s="2">
+        <v>4211112</v>
+      </c>
+      <c r="B41" t="str">
+        <f t="shared" si="0"/>
+        <v>42111120</v>
+      </c>
+      <c r="C41" t="str">
+        <f t="shared" si="1"/>
+        <v>n42111120</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E41" t="s">
+        <v>170</v>
+      </c>
+      <c r="F41" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" s="2">
+        <v>4211129</v>
+      </c>
+      <c r="B42" t="str">
+        <f t="shared" si="0"/>
+        <v>42111290</v>
+      </c>
+      <c r="C42" t="str">
+        <f t="shared" si="1"/>
+        <v>n42111290</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E42" t="s">
+        <v>170</v>
+      </c>
+      <c r="F42" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" s="2">
+        <v>4211122</v>
+      </c>
+      <c r="B43" t="str">
+        <f t="shared" si="0"/>
+        <v>42111220</v>
+      </c>
+      <c r="C43" t="str">
+        <f t="shared" si="1"/>
+        <v>n42111220</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E43" t="s">
+        <v>170</v>
+      </c>
+      <c r="F43" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" s="2">
+        <v>4211219</v>
+      </c>
+      <c r="B44" t="str">
+        <f t="shared" si="0"/>
+        <v>42112190</v>
+      </c>
+      <c r="C44" t="str">
+        <f t="shared" si="1"/>
+        <v>n42112190</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E44" t="s">
+        <v>170</v>
+      </c>
+      <c r="F44" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" s="2">
+        <v>4211212</v>
+      </c>
+      <c r="B45" t="str">
+        <f t="shared" si="0"/>
+        <v>42112120</v>
+      </c>
+      <c r="C45" t="str">
+        <f t="shared" si="1"/>
+        <v>n42112120</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E45" t="s">
+        <v>170</v>
+      </c>
+      <c r="F45" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" s="2">
+        <v>4211229</v>
+      </c>
+      <c r="B46" t="str">
+        <f t="shared" si="0"/>
+        <v>42112290</v>
+      </c>
+      <c r="C46" t="str">
+        <f t="shared" si="1"/>
+        <v>n42112290</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E46" t="s">
+        <v>170</v>
+      </c>
+      <c r="F46" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" s="2">
+        <v>4211222</v>
+      </c>
+      <c r="B47" t="str">
+        <f t="shared" si="0"/>
+        <v>42112220</v>
+      </c>
+      <c r="C47" t="str">
+        <f t="shared" si="1"/>
+        <v>n42112220</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E47" t="s">
+        <v>170</v>
+      </c>
+      <c r="F47" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" s="2">
+        <v>4212119</v>
+      </c>
+      <c r="B48" t="str">
+        <f t="shared" si="0"/>
+        <v>42121190</v>
+      </c>
+      <c r="C48" t="str">
+        <f t="shared" si="1"/>
+        <v>n42121190</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E48" t="s">
+        <v>170</v>
+      </c>
+      <c r="F48" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" s="2">
+        <v>4212112</v>
+      </c>
+      <c r="B49" t="str">
+        <f t="shared" si="0"/>
+        <v>42121120</v>
+      </c>
+      <c r="C49" t="str">
+        <f t="shared" si="1"/>
+        <v>n42121120</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E49" t="s">
+        <v>170</v>
+      </c>
+      <c r="F49" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" s="2">
+        <v>4212129</v>
+      </c>
+      <c r="B50" t="str">
+        <f t="shared" si="0"/>
+        <v>42121290</v>
+      </c>
+      <c r="C50" t="str">
+        <f t="shared" si="1"/>
+        <v>n42121290</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="E50" t="s">
+        <v>170</v>
+      </c>
+      <c r="F50" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" s="2">
+        <v>4212122</v>
+      </c>
+      <c r="B51" t="str">
+        <f t="shared" si="0"/>
+        <v>42121220</v>
+      </c>
+      <c r="C51" t="str">
+        <f t="shared" si="1"/>
+        <v>n42121220</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E51" t="s">
+        <v>170</v>
+      </c>
+      <c r="F51" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" s="2">
+        <v>4212219</v>
+      </c>
+      <c r="B52" t="str">
+        <f t="shared" si="0"/>
+        <v>42122190</v>
+      </c>
+      <c r="C52" t="str">
+        <f t="shared" si="1"/>
+        <v>n42122190</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="E52" t="s">
+        <v>170</v>
+      </c>
+      <c r="F52" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" s="2">
+        <v>4212212</v>
+      </c>
+      <c r="B53" t="str">
+        <f t="shared" si="0"/>
+        <v>42122120</v>
+      </c>
+      <c r="C53" t="str">
+        <f t="shared" si="1"/>
+        <v>n42122120</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E53" t="s">
+        <v>170</v>
+      </c>
+      <c r="F53" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" s="2">
+        <v>4212229</v>
+      </c>
+      <c r="B54" t="str">
+        <f t="shared" si="0"/>
+        <v>42122290</v>
+      </c>
+      <c r="C54" t="str">
+        <f t="shared" si="1"/>
+        <v>n42122290</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="E54" t="s">
+        <v>170</v>
+      </c>
+      <c r="F54" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" s="2">
+        <v>4212222</v>
+      </c>
+      <c r="B55" t="str">
+        <f t="shared" si="0"/>
+        <v>42122220</v>
+      </c>
+      <c r="C55" t="str">
+        <f t="shared" si="1"/>
+        <v>n42122220</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E55" t="s">
+        <v>170</v>
+      </c>
+      <c r="F55" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" s="2">
+        <v>422119</v>
+      </c>
+      <c r="B56" t="str">
+        <f t="shared" si="0"/>
+        <v>42211900</v>
+      </c>
+      <c r="C56" t="str">
+        <f t="shared" si="1"/>
+        <v>n42211900</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E56" t="s">
+        <v>170</v>
+      </c>
+      <c r="F56" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57" s="2">
+        <v>422112</v>
+      </c>
+      <c r="B57" t="str">
+        <f t="shared" si="0"/>
+        <v>42211200</v>
+      </c>
+      <c r="C57" t="str">
+        <f t="shared" si="1"/>
+        <v>n42211200</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="E57" t="s">
+        <v>170</v>
+      </c>
+      <c r="F57" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" s="2">
+        <v>422129</v>
+      </c>
+      <c r="B58" t="str">
+        <f t="shared" si="0"/>
+        <v>42212900</v>
+      </c>
+      <c r="C58" t="str">
+        <f t="shared" si="1"/>
+        <v>n42212900</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E58" t="s">
+        <v>170</v>
+      </c>
+      <c r="F58" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" s="2">
+        <v>422122</v>
+      </c>
+      <c r="B59" t="str">
+        <f t="shared" si="0"/>
+        <v>42212200</v>
+      </c>
+      <c r="C59" t="str">
+        <f t="shared" si="1"/>
+        <v>n42212200</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E59" t="s">
+        <v>170</v>
+      </c>
+      <c r="F59" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" s="2">
+        <v>4222119</v>
+      </c>
+      <c r="B60" t="str">
+        <f t="shared" si="0"/>
+        <v>42221190</v>
+      </c>
+      <c r="C60" t="str">
+        <f t="shared" si="1"/>
+        <v>n42221190</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E60" t="s">
+        <v>170</v>
+      </c>
+      <c r="F60" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" s="2">
+        <v>4222112</v>
+      </c>
+      <c r="B61" t="str">
+        <f t="shared" si="0"/>
+        <v>42221120</v>
+      </c>
+      <c r="C61" t="str">
+        <f t="shared" si="1"/>
+        <v>n42221120</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="E61" t="s">
+        <v>170</v>
+      </c>
+      <c r="F61" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" s="2">
+        <v>42221219</v>
+      </c>
+      <c r="B62" t="str">
+        <f t="shared" si="0"/>
+        <v>42221219</v>
+      </c>
+      <c r="C62" t="str">
+        <f t="shared" si="1"/>
+        <v>n42221219</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E62" t="s">
+        <v>170</v>
+      </c>
+      <c r="F62" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" s="2">
+        <v>42221212</v>
+      </c>
+      <c r="B63" t="str">
+        <f t="shared" si="0"/>
+        <v>42221212</v>
+      </c>
+      <c r="C63" t="str">
+        <f t="shared" si="1"/>
+        <v>n42221212</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E63" t="s">
+        <v>170</v>
+      </c>
+      <c r="F63" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" s="2">
+        <v>42221229</v>
+      </c>
+      <c r="B64" t="str">
+        <f t="shared" si="0"/>
+        <v>42221229</v>
+      </c>
+      <c r="C64" t="str">
+        <f t="shared" si="1"/>
+        <v>n42221229</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E64" t="s">
+        <v>170</v>
+      </c>
+      <c r="F64" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" s="2">
+        <v>42221222</v>
+      </c>
+      <c r="B65" t="str">
+        <f t="shared" si="0"/>
+        <v>42221222</v>
+      </c>
+      <c r="C65" t="str">
+        <f t="shared" si="1"/>
+        <v>n42221222</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="E65" t="s">
+        <v>170</v>
+      </c>
+      <c r="F65" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
+      <c r="A66" s="2">
+        <v>422229</v>
+      </c>
+      <c r="B66" t="str">
+        <f t="shared" si="0"/>
+        <v>42222900</v>
+      </c>
+      <c r="C66" t="str">
+        <f t="shared" si="1"/>
+        <v>n42222900</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E66" t="s">
+        <v>170</v>
+      </c>
+      <c r="F66" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" s="4" customFormat="1">
+      <c r="A67" s="3">
+        <v>422222</v>
+      </c>
+      <c r="B67" s="4" t="str">
+        <f t="shared" ref="B67:B82" si="2">A67&amp;REPT("0",8-LEN(A67))</f>
+        <v>42222200</v>
+      </c>
+      <c r="C67" s="4" t="str">
+        <f t="shared" ref="C67:C82" si="3">_xlfn.CONCAT("n",B67)</f>
+        <v>n42222200</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E67" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="A68" s="2">
+        <v>51</v>
+      </c>
+      <c r="B68" t="str">
+        <f t="shared" si="2"/>
+        <v>51000000</v>
+      </c>
+      <c r="C68" t="str">
+        <f t="shared" si="3"/>
+        <v>n51000000</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E68" t="s">
+        <v>171</v>
+      </c>
+      <c r="F68" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
+      <c r="A69" s="2">
+        <v>5219</v>
+      </c>
+      <c r="B69" t="str">
+        <f t="shared" si="2"/>
+        <v>52190000</v>
+      </c>
+      <c r="C69" t="str">
+        <f t="shared" si="3"/>
+        <v>n52190000</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E69" t="s">
+        <v>171</v>
+      </c>
+      <c r="F69" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
+      <c r="A70" s="2">
+        <v>5212</v>
+      </c>
+      <c r="B70" t="str">
+        <f t="shared" si="2"/>
+        <v>52120000</v>
+      </c>
+      <c r="C70" t="str">
+        <f t="shared" si="3"/>
+        <v>n52120000</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E70" t="s">
+        <v>171</v>
+      </c>
+      <c r="F70" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
+      <c r="A71" s="2">
+        <v>5222</v>
+      </c>
+      <c r="B71" t="str">
+        <f t="shared" si="2"/>
+        <v>52220000</v>
+      </c>
+      <c r="C71" t="str">
+        <f t="shared" si="3"/>
+        <v>n52220000</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E71" t="s">
+        <v>171</v>
+      </c>
+      <c r="F71" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
+      <c r="A72" s="2">
+        <v>5239</v>
+      </c>
+      <c r="B72" t="str">
+        <f t="shared" si="2"/>
+        <v>52390000</v>
+      </c>
+      <c r="C72" t="str">
+        <f t="shared" si="3"/>
+        <v>n52390000</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E72" t="s">
+        <v>171</v>
+      </c>
+      <c r="F72" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
+      <c r="A73" s="2">
+        <v>5232</v>
+      </c>
+      <c r="B73" t="str">
+        <f t="shared" si="2"/>
+        <v>52320000</v>
+      </c>
+      <c r="C73" t="str">
+        <f t="shared" si="3"/>
+        <v>n52320000</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E73" t="s">
+        <v>171</v>
+      </c>
+      <c r="F73" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6">
+      <c r="A74" s="2">
+        <v>539</v>
+      </c>
+      <c r="B74" t="str">
+        <f t="shared" si="2"/>
+        <v>53900000</v>
+      </c>
+      <c r="C74" t="str">
+        <f t="shared" si="3"/>
+        <v>n53900000</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E74" t="s">
+        <v>171</v>
+      </c>
+      <c r="F74" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" s="4" customFormat="1">
+      <c r="A75" s="3">
+        <v>532</v>
+      </c>
+      <c r="B75" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>53200000</v>
+      </c>
+      <c r="C75" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>n53200000</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6">
+      <c r="A76" s="2">
+        <v>61</v>
+      </c>
+      <c r="B76" t="str">
+        <f t="shared" si="2"/>
+        <v>61000000</v>
+      </c>
+      <c r="C76" t="str">
+        <f t="shared" si="3"/>
+        <v>n61000000</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E76" t="s">
+        <v>172</v>
+      </c>
+      <c r="F76" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6">
+      <c r="A77" s="2">
+        <v>6212</v>
+      </c>
+      <c r="B77" t="str">
+        <f t="shared" si="2"/>
+        <v>62120000</v>
+      </c>
+      <c r="C77" t="str">
+        <f t="shared" si="3"/>
+        <v>n62120000</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="E77" t="s">
+        <v>172</v>
+      </c>
+      <c r="F77" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6">
+      <c r="A78" s="2">
+        <v>6229</v>
+      </c>
+      <c r="B78" t="str">
+        <f t="shared" si="2"/>
+        <v>62290000</v>
+      </c>
+      <c r="C78" t="str">
+        <f t="shared" si="3"/>
+        <v>n62290000</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E78" t="s">
+        <v>172</v>
+      </c>
+      <c r="F78" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6">
+      <c r="A79" s="2">
+        <v>6222</v>
+      </c>
+      <c r="B79" t="str">
+        <f t="shared" si="2"/>
+        <v>62220000</v>
+      </c>
+      <c r="C79" t="str">
+        <f t="shared" si="3"/>
+        <v>n62220000</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E79" t="s">
+        <v>172</v>
+      </c>
+      <c r="F79" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6">
+      <c r="A80" s="2">
+        <v>639</v>
+      </c>
+      <c r="B80" t="str">
+        <f t="shared" si="2"/>
+        <v>63900000</v>
+      </c>
+      <c r="C80" t="str">
+        <f t="shared" si="3"/>
+        <v>n63900000</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="E80" t="s">
+        <v>172</v>
+      </c>
+      <c r="F80" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" s="4" customFormat="1">
+      <c r="A81" s="3">
+        <v>632</v>
+      </c>
+      <c r="B81" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>63200000</v>
+      </c>
+      <c r="C81" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>n63200000</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E81" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6">
+      <c r="A82" s="2">
+        <v>7</v>
+      </c>
+      <c r="B82" t="str">
+        <f t="shared" si="2"/>
+        <v>70000000</v>
+      </c>
+      <c r="C82" t="str">
+        <f t="shared" si="3"/>
+        <v>n70000000</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E82" t="s">
+        <v>174</v>
+      </c>
+      <c r="F82" t="s">
+        <v>174</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1" xr:uid="{853D7656-B308-4E3A-9467-98AD8F1F4D68}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{853D7656-B308-4E3A-9467-98AD8F1F4D68}">
   <dimension ref="A1:F82"/>
   <sheetFormatPr defaultRowHeight="14.5"/>

</xml_diff>

<commit_message>
Added some potential changes to try speeding up global geotif creation. Haven't tested them at all. Left as TODOs. Tried running zonal stats on the mega-zarr but got that float32/fill value error. I think I need to rethink the zarr creation step to avoid that fillvalue hack.
</commit_message>
<xml_diff>
--- a/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
+++ b/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
@@ -1,28 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIS\git\AFOLU_GHG_flux_model\src\LULUCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E38FF9-D75E-4C6D-A6A6-5997748DFEA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54522CD7-E9E1-451D-8CB6-990F926B2213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-9795" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="v030_20250430" sheetId="1" r:id="rId1"/>
     <sheet name="v040_20250713" sheetId="3" r:id="rId2"/>
     <sheet name="v042_20250805" sheetId="2" r:id="rId3"/>
+    <sheet name="v102_20251027" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">v040_20250713!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">v042_20250805!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">v102_20251027!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="190">
   <si>
     <t>meaning</t>
   </si>
@@ -568,6 +569,51 @@
   </si>
   <si>
     <t>no_flux</t>
+  </si>
+  <si>
+    <t>Permanent loss of mangroves to water</t>
+  </si>
+  <si>
+    <t>Permanent loss of mangroves to cropland</t>
+  </si>
+  <si>
+    <t>Permanent loss of mangroves to settlement</t>
+  </si>
+  <si>
+    <t>Permanent loss of mangroves to short vegetation</t>
+  </si>
+  <si>
+    <t>Permanent loss of mangroves to tall vegetation</t>
+  </si>
+  <si>
+    <t>Permanent loss of mangroves to anything else</t>
+  </si>
+  <si>
+    <t>Temporary loss of mangroves</t>
+  </si>
+  <si>
+    <t>Mangrove remaining mangrove + temp loss in interval</t>
+  </si>
+  <si>
+    <t>Mangrove remaining mangrove, no loss in interval</t>
+  </si>
+  <si>
+    <t>Before mangrove gain (mangrove mask)</t>
+  </si>
+  <si>
+    <t>Non-mangrove remaining non-mangrove (mangrove mask)</t>
+  </si>
+  <si>
+    <t>After permanent mangrove loss (mangrove mask)</t>
+  </si>
+  <si>
+    <t>mangrove_other</t>
+  </si>
+  <si>
+    <t>Gain of mangroves + temp loss in interval</t>
+  </si>
+  <si>
+    <t>Gain of mangroves, no loss in interval</t>
   </si>
 </sst>
 </file>
@@ -627,7 +673,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -637,6 +683,11 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5482,4 +5533,2134 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A7BB84B-4BF3-4978-BFCA-0C4F8A30C442}">
+  <dimension ref="A1:F96"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="132.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="5">
+        <v>111</v>
+      </c>
+      <c r="B2" s="6" t="str">
+        <f t="shared" ref="B2:B3" si="0">A2&amp;REPT("0",8-LEN(A2))</f>
+        <v>11100000</v>
+      </c>
+      <c r="C2" s="6" t="str">
+        <f t="shared" ref="C2:C3" si="1">_xlfn.CONCAT("n",B2)</f>
+        <v>n11100000</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="5">
+        <v>112</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>11200000</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v>n11200000</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="6" customFormat="1">
+      <c r="A4" s="5">
+        <v>122</v>
+      </c>
+      <c r="B4" s="6" t="str">
+        <f>A4&amp;REPT("0",8-LEN(A4))</f>
+        <v>12200000</v>
+      </c>
+      <c r="C4" s="6" t="str">
+        <f>_xlfn.CONCAT("n",B4)</f>
+        <v>n12200000</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="6" customFormat="1">
+      <c r="A5" s="5">
+        <v>123</v>
+      </c>
+      <c r="B5" s="6" t="str">
+        <f t="shared" ref="B5:B68" si="2">A5&amp;REPT("0",8-LEN(A5))</f>
+        <v>12300000</v>
+      </c>
+      <c r="C5" s="6" t="str">
+        <f t="shared" ref="C5:C68" si="3">_xlfn.CONCAT("n",B5)</f>
+        <v>n12300000</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="6" customFormat="1">
+      <c r="A6" s="5">
+        <v>124</v>
+      </c>
+      <c r="B6" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>12400000</v>
+      </c>
+      <c r="C6" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n12400000</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="6" customFormat="1">
+      <c r="A7" s="5">
+        <v>125</v>
+      </c>
+      <c r="B7" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>12500000</v>
+      </c>
+      <c r="C7" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n12500000</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="6" customFormat="1">
+      <c r="A8" s="5">
+        <v>126</v>
+      </c>
+      <c r="B8" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>12600000</v>
+      </c>
+      <c r="C8" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n12600000</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="6" customFormat="1">
+      <c r="A9" s="5">
+        <v>127</v>
+      </c>
+      <c r="B9" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>12700000</v>
+      </c>
+      <c r="C9" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n12700000</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="6" customFormat="1">
+      <c r="A10" s="5">
+        <v>121</v>
+      </c>
+      <c r="B10" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>12100000</v>
+      </c>
+      <c r="C10" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n12100000</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="6" customFormat="1">
+      <c r="A11" s="5">
+        <v>131</v>
+      </c>
+      <c r="B11" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>13100000</v>
+      </c>
+      <c r="C11" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n13100000</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="6" customFormat="1">
+      <c r="A12" s="5">
+        <v>132</v>
+      </c>
+      <c r="B12" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>13200000</v>
+      </c>
+      <c r="C12" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n13200000</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F12" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="6" customFormat="1">
+      <c r="A13" s="5">
+        <v>100</v>
+      </c>
+      <c r="B13" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>10000000</v>
+      </c>
+      <c r="C13" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n10000000</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="6" customFormat="1">
+      <c r="A14" s="5">
+        <v>101</v>
+      </c>
+      <c r="B14" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>10100000</v>
+      </c>
+      <c r="C14" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n10100000</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="4" customFormat="1">
+      <c r="A15" s="3">
+        <v>102</v>
+      </c>
+      <c r="B15" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>10200000</v>
+      </c>
+      <c r="C15" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>n10200000</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="6" customFormat="1">
+      <c r="A16" s="5">
+        <v>211</v>
+      </c>
+      <c r="B16" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>21100000</v>
+      </c>
+      <c r="C16" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n21100000</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" t="s">
+        <v>170</v>
+      </c>
+      <c r="F16" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" s="6" customFormat="1">
+      <c r="A17" s="5">
+        <v>212</v>
+      </c>
+      <c r="B17" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>21200000</v>
+      </c>
+      <c r="C17" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n21200000</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E17" t="s">
+        <v>170</v>
+      </c>
+      <c r="F17" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="6" customFormat="1">
+      <c r="A18" s="5">
+        <v>221</v>
+      </c>
+      <c r="B18" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>22100000</v>
+      </c>
+      <c r="C18" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n22100000</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E18" t="s">
+        <v>170</v>
+      </c>
+      <c r="F18" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="4" customFormat="1">
+      <c r="A19" s="3">
+        <v>222</v>
+      </c>
+      <c r="B19" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>22200000</v>
+      </c>
+      <c r="C19" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>n22200000</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="6" customFormat="1">
+      <c r="A20" s="2">
+        <v>3119</v>
+      </c>
+      <c r="B20" t="str">
+        <f t="shared" si="2"/>
+        <v>31190000</v>
+      </c>
+      <c r="C20" t="str">
+        <f t="shared" si="3"/>
+        <v>n31190000</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E20" t="s">
+        <v>170</v>
+      </c>
+      <c r="F20" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" s="6" customFormat="1">
+      <c r="A21" s="2">
+        <v>3112</v>
+      </c>
+      <c r="B21" t="str">
+        <f t="shared" si="2"/>
+        <v>31120000</v>
+      </c>
+      <c r="C21" t="str">
+        <f t="shared" si="3"/>
+        <v>n31120000</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E21" t="s">
+        <v>170</v>
+      </c>
+      <c r="F21" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="6" customFormat="1">
+      <c r="A22" s="2">
+        <v>312119</v>
+      </c>
+      <c r="B22" t="str">
+        <f t="shared" si="2"/>
+        <v>31211900</v>
+      </c>
+      <c r="C22" t="str">
+        <f t="shared" si="3"/>
+        <v>n31211900</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E22" t="s">
+        <v>170</v>
+      </c>
+      <c r="F22" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" s="6" customFormat="1">
+      <c r="A23" s="2">
+        <v>312112</v>
+      </c>
+      <c r="B23" t="str">
+        <f t="shared" si="2"/>
+        <v>31211200</v>
+      </c>
+      <c r="C23" t="str">
+        <f t="shared" si="3"/>
+        <v>n31211200</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E23" t="s">
+        <v>170</v>
+      </c>
+      <c r="F23" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" s="6" customFormat="1">
+      <c r="A24" s="2">
+        <v>312129</v>
+      </c>
+      <c r="B24" t="str">
+        <f t="shared" si="2"/>
+        <v>31212900</v>
+      </c>
+      <c r="C24" t="str">
+        <f t="shared" si="3"/>
+        <v>n31212900</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E24" t="s">
+        <v>170</v>
+      </c>
+      <c r="F24" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" s="6" customFormat="1">
+      <c r="A25" s="2">
+        <v>312122</v>
+      </c>
+      <c r="B25" t="str">
+        <f t="shared" si="2"/>
+        <v>31212200</v>
+      </c>
+      <c r="C25" t="str">
+        <f t="shared" si="3"/>
+        <v>n31212200</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E25" t="s">
+        <v>170</v>
+      </c>
+      <c r="F25" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" s="6" customFormat="1">
+      <c r="A26" s="2">
+        <v>312219</v>
+      </c>
+      <c r="B26" t="str">
+        <f t="shared" si="2"/>
+        <v>31221900</v>
+      </c>
+      <c r="C26" t="str">
+        <f t="shared" si="3"/>
+        <v>n31221900</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E26" t="s">
+        <v>170</v>
+      </c>
+      <c r="F26" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" s="6" customFormat="1">
+      <c r="A27" s="2">
+        <v>312212</v>
+      </c>
+      <c r="B27" t="str">
+        <f t="shared" si="2"/>
+        <v>31221200</v>
+      </c>
+      <c r="C27" t="str">
+        <f t="shared" si="3"/>
+        <v>n31221200</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E27" t="s">
+        <v>170</v>
+      </c>
+      <c r="F27" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" s="6" customFormat="1">
+      <c r="A28" s="2">
+        <v>312229</v>
+      </c>
+      <c r="B28" t="str">
+        <f t="shared" si="2"/>
+        <v>31222900</v>
+      </c>
+      <c r="C28" t="str">
+        <f t="shared" si="3"/>
+        <v>n31222900</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E28" t="s">
+        <v>170</v>
+      </c>
+      <c r="F28" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" s="6" customFormat="1">
+      <c r="A29" s="2">
+        <v>312222</v>
+      </c>
+      <c r="B29" t="str">
+        <f t="shared" si="2"/>
+        <v>31222200</v>
+      </c>
+      <c r="C29" t="str">
+        <f t="shared" si="3"/>
+        <v>n31222200</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E29" t="s">
+        <v>170</v>
+      </c>
+      <c r="F29" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" s="6" customFormat="1">
+      <c r="A30" s="2">
+        <v>312319</v>
+      </c>
+      <c r="B30" t="str">
+        <f t="shared" si="2"/>
+        <v>31231900</v>
+      </c>
+      <c r="C30" t="str">
+        <f t="shared" si="3"/>
+        <v>n31231900</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E30" t="s">
+        <v>170</v>
+      </c>
+      <c r="F30" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" s="6" customFormat="1">
+      <c r="A31" s="2">
+        <v>312312</v>
+      </c>
+      <c r="B31" t="str">
+        <f t="shared" si="2"/>
+        <v>31231200</v>
+      </c>
+      <c r="C31" t="str">
+        <f t="shared" si="3"/>
+        <v>n31231200</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E31" t="s">
+        <v>170</v>
+      </c>
+      <c r="F31" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" s="6" customFormat="1">
+      <c r="A32" s="2">
+        <v>312329</v>
+      </c>
+      <c r="B32" t="str">
+        <f t="shared" si="2"/>
+        <v>31232900</v>
+      </c>
+      <c r="C32" t="str">
+        <f t="shared" si="3"/>
+        <v>n31232900</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E32" t="s">
+        <v>170</v>
+      </c>
+      <c r="F32" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" s="6" customFormat="1">
+      <c r="A33" s="2">
+        <v>312322</v>
+      </c>
+      <c r="B33" t="str">
+        <f t="shared" si="2"/>
+        <v>31232200</v>
+      </c>
+      <c r="C33" t="str">
+        <f t="shared" si="3"/>
+        <v>n31232200</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E33" t="s">
+        <v>170</v>
+      </c>
+      <c r="F33" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" s="6" customFormat="1">
+      <c r="A34" s="2">
+        <v>312412</v>
+      </c>
+      <c r="B34" t="str">
+        <f t="shared" si="2"/>
+        <v>31241200</v>
+      </c>
+      <c r="C34" t="str">
+        <f t="shared" si="3"/>
+        <v>n31241200</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E34" t="s">
+        <v>170</v>
+      </c>
+      <c r="F34" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" s="6" customFormat="1">
+      <c r="A35" s="2">
+        <v>312422</v>
+      </c>
+      <c r="B35" t="str">
+        <f t="shared" si="2"/>
+        <v>31242200</v>
+      </c>
+      <c r="C35" t="str">
+        <f t="shared" si="3"/>
+        <v>n31242200</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E35" t="s">
+        <v>170</v>
+      </c>
+      <c r="F35" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" s="6" customFormat="1">
+      <c r="A36" s="2">
+        <v>32119</v>
+      </c>
+      <c r="B36" t="str">
+        <f t="shared" si="2"/>
+        <v>32119000</v>
+      </c>
+      <c r="C36" t="str">
+        <f t="shared" si="3"/>
+        <v>n32119000</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E36" t="s">
+        <v>170</v>
+      </c>
+      <c r="F36" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" s="6" customFormat="1">
+      <c r="A37" s="2">
+        <v>32112</v>
+      </c>
+      <c r="B37" t="str">
+        <f t="shared" si="2"/>
+        <v>32112000</v>
+      </c>
+      <c r="C37" t="str">
+        <f t="shared" si="3"/>
+        <v>n32112000</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E37" t="s">
+        <v>170</v>
+      </c>
+      <c r="F37" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" s="6" customFormat="1">
+      <c r="A38" s="2">
+        <v>321219</v>
+      </c>
+      <c r="B38" t="str">
+        <f t="shared" si="2"/>
+        <v>32121900</v>
+      </c>
+      <c r="C38" t="str">
+        <f t="shared" si="3"/>
+        <v>n32121900</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E38" t="s">
+        <v>170</v>
+      </c>
+      <c r="F38" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" s="6" customFormat="1">
+      <c r="A39" s="2">
+        <v>321212</v>
+      </c>
+      <c r="B39" t="str">
+        <f t="shared" si="2"/>
+        <v>32121200</v>
+      </c>
+      <c r="C39" t="str">
+        <f t="shared" si="3"/>
+        <v>n32121200</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E39" t="s">
+        <v>170</v>
+      </c>
+      <c r="F39" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" s="6" customFormat="1">
+      <c r="A40" s="2">
+        <v>321229</v>
+      </c>
+      <c r="B40" t="str">
+        <f t="shared" si="2"/>
+        <v>32122900</v>
+      </c>
+      <c r="C40" t="str">
+        <f t="shared" si="3"/>
+        <v>n32122900</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E40" t="s">
+        <v>170</v>
+      </c>
+      <c r="F40" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" s="6" customFormat="1">
+      <c r="A41" s="2">
+        <v>321222</v>
+      </c>
+      <c r="B41" t="str">
+        <f t="shared" si="2"/>
+        <v>32122200</v>
+      </c>
+      <c r="C41" t="str">
+        <f t="shared" si="3"/>
+        <v>n32122200</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E41" t="s">
+        <v>170</v>
+      </c>
+      <c r="F41" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" s="6" customFormat="1">
+      <c r="A42" s="2">
+        <v>32139</v>
+      </c>
+      <c r="B42" t="str">
+        <f t="shared" si="2"/>
+        <v>32139000</v>
+      </c>
+      <c r="C42" t="str">
+        <f t="shared" si="3"/>
+        <v>n32139000</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E42" t="s">
+        <v>170</v>
+      </c>
+      <c r="F42" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" s="6" customFormat="1">
+      <c r="A43" s="2">
+        <v>32132</v>
+      </c>
+      <c r="B43" t="str">
+        <f t="shared" si="2"/>
+        <v>32132000</v>
+      </c>
+      <c r="C43" t="str">
+        <f t="shared" si="3"/>
+        <v>n32132000</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E43" t="s">
+        <v>170</v>
+      </c>
+      <c r="F43" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" s="6" customFormat="1">
+      <c r="A44" s="2">
+        <v>32142</v>
+      </c>
+      <c r="B44" t="str">
+        <f t="shared" si="2"/>
+        <v>32142000</v>
+      </c>
+      <c r="C44" t="str">
+        <f t="shared" si="3"/>
+        <v>n32142000</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E44" t="s">
+        <v>170</v>
+      </c>
+      <c r="F44" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" s="6" customFormat="1">
+      <c r="A45" s="2">
+        <v>32219</v>
+      </c>
+      <c r="B45" t="str">
+        <f t="shared" si="2"/>
+        <v>32219000</v>
+      </c>
+      <c r="C45" t="str">
+        <f t="shared" si="3"/>
+        <v>n32219000</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E45" t="s">
+        <v>170</v>
+      </c>
+      <c r="F45" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" s="6" customFormat="1">
+      <c r="A46" s="2">
+        <v>32212</v>
+      </c>
+      <c r="B46" t="str">
+        <f t="shared" si="2"/>
+        <v>32212000</v>
+      </c>
+      <c r="C46" t="str">
+        <f t="shared" si="3"/>
+        <v>n32212000</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E46" t="s">
+        <v>170</v>
+      </c>
+      <c r="F46" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" s="6" customFormat="1">
+      <c r="A47" s="2">
+        <v>32229</v>
+      </c>
+      <c r="B47" t="str">
+        <f t="shared" si="2"/>
+        <v>32229000</v>
+      </c>
+      <c r="C47" t="str">
+        <f t="shared" si="3"/>
+        <v>n32229000</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E47" t="s">
+        <v>170</v>
+      </c>
+      <c r="F47" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" s="6" customFormat="1">
+      <c r="A48" s="2">
+        <v>32222</v>
+      </c>
+      <c r="B48" t="str">
+        <f t="shared" si="2"/>
+        <v>32222000</v>
+      </c>
+      <c r="C48" t="str">
+        <f t="shared" si="3"/>
+        <v>n32222000</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E48" t="s">
+        <v>170</v>
+      </c>
+      <c r="F48" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" s="6" customFormat="1">
+      <c r="A49" s="2">
+        <v>32239</v>
+      </c>
+      <c r="B49" t="str">
+        <f t="shared" si="2"/>
+        <v>32239000</v>
+      </c>
+      <c r="C49" t="str">
+        <f t="shared" si="3"/>
+        <v>n32239000</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E49" t="s">
+        <v>170</v>
+      </c>
+      <c r="F49" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" s="6" customFormat="1">
+      <c r="A50" s="2">
+        <v>32232</v>
+      </c>
+      <c r="B50" t="str">
+        <f t="shared" si="2"/>
+        <v>32232000</v>
+      </c>
+      <c r="C50" t="str">
+        <f t="shared" si="3"/>
+        <v>n32232000</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E50" t="s">
+        <v>170</v>
+      </c>
+      <c r="F50" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" s="4" customFormat="1">
+      <c r="A51" s="3">
+        <v>32242</v>
+      </c>
+      <c r="B51" s="4" t="str">
+        <f t="shared" si="2"/>
+        <v>32242000</v>
+      </c>
+      <c r="C51" s="4" t="str">
+        <f t="shared" si="3"/>
+        <v>n32242000</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" s="6" customFormat="1">
+      <c r="A52" s="5">
+        <v>419</v>
+      </c>
+      <c r="B52" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>41900000</v>
+      </c>
+      <c r="C52" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n41900000</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" s="6" customFormat="1">
+      <c r="A53" s="5">
+        <v>412</v>
+      </c>
+      <c r="B53" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>41200000</v>
+      </c>
+      <c r="C53" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>n41200000</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F53" s="6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" s="6" customFormat="1">
+      <c r="A54" s="2">
+        <v>4211119</v>
+      </c>
+      <c r="B54" t="str">
+        <f t="shared" si="2"/>
+        <v>42111190</v>
+      </c>
+      <c r="C54" t="str">
+        <f t="shared" si="3"/>
+        <v>n42111190</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E54" t="s">
+        <v>170</v>
+      </c>
+      <c r="F54" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" s="6" customFormat="1">
+      <c r="A55" s="2">
+        <v>4211112</v>
+      </c>
+      <c r="B55" t="str">
+        <f t="shared" si="2"/>
+        <v>42111120</v>
+      </c>
+      <c r="C55" t="str">
+        <f t="shared" si="3"/>
+        <v>n42111120</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E55" t="s">
+        <v>170</v>
+      </c>
+      <c r="F55" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" s="6" customFormat="1">
+      <c r="A56" s="2">
+        <v>4211129</v>
+      </c>
+      <c r="B56" t="str">
+        <f t="shared" si="2"/>
+        <v>42111290</v>
+      </c>
+      <c r="C56" t="str">
+        <f t="shared" si="3"/>
+        <v>n42111290</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E56" t="s">
+        <v>170</v>
+      </c>
+      <c r="F56" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" s="6" customFormat="1">
+      <c r="A57" s="2">
+        <v>4211122</v>
+      </c>
+      <c r="B57" t="str">
+        <f t="shared" si="2"/>
+        <v>42111220</v>
+      </c>
+      <c r="C57" t="str">
+        <f t="shared" si="3"/>
+        <v>n42111220</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E57" t="s">
+        <v>170</v>
+      </c>
+      <c r="F57" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" s="6" customFormat="1">
+      <c r="A58" s="2">
+        <v>4211219</v>
+      </c>
+      <c r="B58" t="str">
+        <f t="shared" si="2"/>
+        <v>42112190</v>
+      </c>
+      <c r="C58" t="str">
+        <f t="shared" si="3"/>
+        <v>n42112190</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E58" t="s">
+        <v>170</v>
+      </c>
+      <c r="F58" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" s="6" customFormat="1">
+      <c r="A59" s="2">
+        <v>4211212</v>
+      </c>
+      <c r="B59" t="str">
+        <f t="shared" si="2"/>
+        <v>42112120</v>
+      </c>
+      <c r="C59" t="str">
+        <f t="shared" si="3"/>
+        <v>n42112120</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E59" t="s">
+        <v>170</v>
+      </c>
+      <c r="F59" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" s="6" customFormat="1">
+      <c r="A60" s="2">
+        <v>4211229</v>
+      </c>
+      <c r="B60" t="str">
+        <f t="shared" si="2"/>
+        <v>42112290</v>
+      </c>
+      <c r="C60" t="str">
+        <f t="shared" si="3"/>
+        <v>n42112290</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E60" t="s">
+        <v>170</v>
+      </c>
+      <c r="F60" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" s="6" customFormat="1">
+      <c r="A61" s="2">
+        <v>4211222</v>
+      </c>
+      <c r="B61" t="str">
+        <f t="shared" si="2"/>
+        <v>42112220</v>
+      </c>
+      <c r="C61" t="str">
+        <f t="shared" si="3"/>
+        <v>n42112220</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E61" t="s">
+        <v>170</v>
+      </c>
+      <c r="F61" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" s="6" customFormat="1">
+      <c r="A62" s="2">
+        <v>4212119</v>
+      </c>
+      <c r="B62" t="str">
+        <f t="shared" si="2"/>
+        <v>42121190</v>
+      </c>
+      <c r="C62" t="str">
+        <f t="shared" si="3"/>
+        <v>n42121190</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E62" t="s">
+        <v>170</v>
+      </c>
+      <c r="F62" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" s="6" customFormat="1">
+      <c r="A63" s="2">
+        <v>4212112</v>
+      </c>
+      <c r="B63" t="str">
+        <f t="shared" si="2"/>
+        <v>42121120</v>
+      </c>
+      <c r="C63" t="str">
+        <f t="shared" si="3"/>
+        <v>n42121120</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E63" t="s">
+        <v>170</v>
+      </c>
+      <c r="F63" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" s="6" customFormat="1">
+      <c r="A64" s="2">
+        <v>4212129</v>
+      </c>
+      <c r="B64" t="str">
+        <f t="shared" si="2"/>
+        <v>42121290</v>
+      </c>
+      <c r="C64" t="str">
+        <f t="shared" si="3"/>
+        <v>n42121290</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="E64" t="s">
+        <v>170</v>
+      </c>
+      <c r="F64" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" s="6" customFormat="1">
+      <c r="A65" s="2">
+        <v>4212122</v>
+      </c>
+      <c r="B65" t="str">
+        <f t="shared" si="2"/>
+        <v>42121220</v>
+      </c>
+      <c r="C65" t="str">
+        <f t="shared" si="3"/>
+        <v>n42121220</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E65" t="s">
+        <v>170</v>
+      </c>
+      <c r="F65" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" s="6" customFormat="1">
+      <c r="A66" s="2">
+        <v>4212219</v>
+      </c>
+      <c r="B66" t="str">
+        <f t="shared" si="2"/>
+        <v>42122190</v>
+      </c>
+      <c r="C66" t="str">
+        <f t="shared" si="3"/>
+        <v>n42122190</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="E66" t="s">
+        <v>170</v>
+      </c>
+      <c r="F66" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" s="6" customFormat="1">
+      <c r="A67" s="2">
+        <v>4212212</v>
+      </c>
+      <c r="B67" t="str">
+        <f t="shared" si="2"/>
+        <v>42122120</v>
+      </c>
+      <c r="C67" t="str">
+        <f t="shared" si="3"/>
+        <v>n42122120</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E67" t="s">
+        <v>170</v>
+      </c>
+      <c r="F67" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" s="6" customFormat="1">
+      <c r="A68" s="2">
+        <v>4212229</v>
+      </c>
+      <c r="B68" t="str">
+        <f t="shared" si="2"/>
+        <v>42122290</v>
+      </c>
+      <c r="C68" t="str">
+        <f t="shared" si="3"/>
+        <v>n42122290</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="E68" t="s">
+        <v>170</v>
+      </c>
+      <c r="F68" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" s="6" customFormat="1">
+      <c r="A69" s="2">
+        <v>4212222</v>
+      </c>
+      <c r="B69" t="str">
+        <f t="shared" ref="B69:B96" si="4">A69&amp;REPT("0",8-LEN(A69))</f>
+        <v>42122220</v>
+      </c>
+      <c r="C69" t="str">
+        <f t="shared" ref="C69:C96" si="5">_xlfn.CONCAT("n",B69)</f>
+        <v>n42122220</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E69" t="s">
+        <v>170</v>
+      </c>
+      <c r="F69" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" s="6" customFormat="1">
+      <c r="A70" s="2">
+        <v>422119</v>
+      </c>
+      <c r="B70" t="str">
+        <f t="shared" si="4"/>
+        <v>42211900</v>
+      </c>
+      <c r="C70" t="str">
+        <f t="shared" si="5"/>
+        <v>n42211900</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E70" t="s">
+        <v>170</v>
+      </c>
+      <c r="F70" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" s="6" customFormat="1">
+      <c r="A71" s="2">
+        <v>422112</v>
+      </c>
+      <c r="B71" t="str">
+        <f t="shared" si="4"/>
+        <v>42211200</v>
+      </c>
+      <c r="C71" t="str">
+        <f t="shared" si="5"/>
+        <v>n42211200</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="E71" t="s">
+        <v>170</v>
+      </c>
+      <c r="F71" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" s="6" customFormat="1">
+      <c r="A72" s="2">
+        <v>422129</v>
+      </c>
+      <c r="B72" t="str">
+        <f t="shared" si="4"/>
+        <v>42212900</v>
+      </c>
+      <c r="C72" t="str">
+        <f t="shared" si="5"/>
+        <v>n42212900</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E72" t="s">
+        <v>170</v>
+      </c>
+      <c r="F72" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" s="6" customFormat="1">
+      <c r="A73" s="2">
+        <v>422122</v>
+      </c>
+      <c r="B73" t="str">
+        <f t="shared" si="4"/>
+        <v>42212200</v>
+      </c>
+      <c r="C73" t="str">
+        <f t="shared" si="5"/>
+        <v>n42212200</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E73" t="s">
+        <v>170</v>
+      </c>
+      <c r="F73" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" s="6" customFormat="1">
+      <c r="A74" s="2">
+        <v>4222119</v>
+      </c>
+      <c r="B74" t="str">
+        <f t="shared" si="4"/>
+        <v>42221190</v>
+      </c>
+      <c r="C74" t="str">
+        <f t="shared" si="5"/>
+        <v>n42221190</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E74" t="s">
+        <v>170</v>
+      </c>
+      <c r="F74" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" s="6" customFormat="1">
+      <c r="A75" s="2">
+        <v>4222112</v>
+      </c>
+      <c r="B75" t="str">
+        <f t="shared" si="4"/>
+        <v>42221120</v>
+      </c>
+      <c r="C75" t="str">
+        <f t="shared" si="5"/>
+        <v>n42221120</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="E75" t="s">
+        <v>170</v>
+      </c>
+      <c r="F75" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" s="6" customFormat="1">
+      <c r="A76" s="2">
+        <v>42221219</v>
+      </c>
+      <c r="B76" t="str">
+        <f t="shared" si="4"/>
+        <v>42221219</v>
+      </c>
+      <c r="C76" t="str">
+        <f t="shared" si="5"/>
+        <v>n42221219</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E76" t="s">
+        <v>170</v>
+      </c>
+      <c r="F76" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" s="6" customFormat="1">
+      <c r="A77" s="2">
+        <v>42221212</v>
+      </c>
+      <c r="B77" t="str">
+        <f t="shared" si="4"/>
+        <v>42221212</v>
+      </c>
+      <c r="C77" t="str">
+        <f t="shared" si="5"/>
+        <v>n42221212</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E77" t="s">
+        <v>170</v>
+      </c>
+      <c r="F77" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" s="6" customFormat="1">
+      <c r="A78" s="2">
+        <v>42221229</v>
+      </c>
+      <c r="B78" t="str">
+        <f t="shared" si="4"/>
+        <v>42221229</v>
+      </c>
+      <c r="C78" t="str">
+        <f t="shared" si="5"/>
+        <v>n42221229</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E78" t="s">
+        <v>170</v>
+      </c>
+      <c r="F78" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" s="6" customFormat="1">
+      <c r="A79" s="2">
+        <v>42221222</v>
+      </c>
+      <c r="B79" t="str">
+        <f t="shared" si="4"/>
+        <v>42221222</v>
+      </c>
+      <c r="C79" t="str">
+        <f t="shared" si="5"/>
+        <v>n42221222</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="E79" t="s">
+        <v>170</v>
+      </c>
+      <c r="F79" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" s="6" customFormat="1">
+      <c r="A80" s="2">
+        <v>422229</v>
+      </c>
+      <c r="B80" t="str">
+        <f t="shared" si="4"/>
+        <v>42222900</v>
+      </c>
+      <c r="C80" t="str">
+        <f t="shared" si="5"/>
+        <v>n42222900</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E80" t="s">
+        <v>170</v>
+      </c>
+      <c r="F80" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" s="6" customFormat="1">
+      <c r="A81" s="3">
+        <v>422222</v>
+      </c>
+      <c r="B81" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>42222200</v>
+      </c>
+      <c r="C81" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>n42222200</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E81" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" s="6" customFormat="1">
+      <c r="A82" s="2">
+        <v>51</v>
+      </c>
+      <c r="B82" t="str">
+        <f t="shared" si="4"/>
+        <v>51000000</v>
+      </c>
+      <c r="C82" t="str">
+        <f t="shared" si="5"/>
+        <v>n51000000</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E82" t="s">
+        <v>171</v>
+      </c>
+      <c r="F82" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" s="6" customFormat="1">
+      <c r="A83" s="2">
+        <v>5219</v>
+      </c>
+      <c r="B83" t="str">
+        <f t="shared" si="4"/>
+        <v>52190000</v>
+      </c>
+      <c r="C83" t="str">
+        <f t="shared" si="5"/>
+        <v>n52190000</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E83" t="s">
+        <v>171</v>
+      </c>
+      <c r="F83" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" s="6" customFormat="1">
+      <c r="A84" s="2">
+        <v>5212</v>
+      </c>
+      <c r="B84" t="str">
+        <f t="shared" si="4"/>
+        <v>52120000</v>
+      </c>
+      <c r="C84" t="str">
+        <f t="shared" si="5"/>
+        <v>n52120000</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E84" t="s">
+        <v>171</v>
+      </c>
+      <c r="F84" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6">
+      <c r="A85" s="2">
+        <v>5222</v>
+      </c>
+      <c r="B85" t="str">
+        <f t="shared" si="4"/>
+        <v>52220000</v>
+      </c>
+      <c r="C85" t="str">
+        <f t="shared" si="5"/>
+        <v>n52220000</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E85" t="s">
+        <v>171</v>
+      </c>
+      <c r="F85" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6">
+      <c r="A86" s="2">
+        <v>5239</v>
+      </c>
+      <c r="B86" t="str">
+        <f t="shared" si="4"/>
+        <v>52390000</v>
+      </c>
+      <c r="C86" t="str">
+        <f t="shared" si="5"/>
+        <v>n52390000</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E86" t="s">
+        <v>171</v>
+      </c>
+      <c r="F86" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6">
+      <c r="A87" s="2">
+        <v>5232</v>
+      </c>
+      <c r="B87" t="str">
+        <f t="shared" si="4"/>
+        <v>52320000</v>
+      </c>
+      <c r="C87" t="str">
+        <f t="shared" si="5"/>
+        <v>n52320000</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E87" t="s">
+        <v>171</v>
+      </c>
+      <c r="F87" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6">
+      <c r="A88" s="2">
+        <v>539</v>
+      </c>
+      <c r="B88" t="str">
+        <f t="shared" si="4"/>
+        <v>53900000</v>
+      </c>
+      <c r="C88" t="str">
+        <f t="shared" si="5"/>
+        <v>n53900000</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E88" t="s">
+        <v>171</v>
+      </c>
+      <c r="F88" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6">
+      <c r="A89" s="3">
+        <v>532</v>
+      </c>
+      <c r="B89" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>53200000</v>
+      </c>
+      <c r="C89" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>n53200000</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6">
+      <c r="A90" s="2">
+        <v>61</v>
+      </c>
+      <c r="B90" t="str">
+        <f t="shared" si="4"/>
+        <v>61000000</v>
+      </c>
+      <c r="C90" t="str">
+        <f t="shared" si="5"/>
+        <v>n61000000</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E90" t="s">
+        <v>172</v>
+      </c>
+      <c r="F90" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6">
+      <c r="A91" s="2">
+        <v>6212</v>
+      </c>
+      <c r="B91" t="str">
+        <f t="shared" si="4"/>
+        <v>62120000</v>
+      </c>
+      <c r="C91" t="str">
+        <f t="shared" si="5"/>
+        <v>n62120000</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="E91" t="s">
+        <v>172</v>
+      </c>
+      <c r="F91" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6">
+      <c r="A92" s="2">
+        <v>6229</v>
+      </c>
+      <c r="B92" t="str">
+        <f t="shared" si="4"/>
+        <v>62290000</v>
+      </c>
+      <c r="C92" t="str">
+        <f t="shared" si="5"/>
+        <v>n62290000</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E92" t="s">
+        <v>172</v>
+      </c>
+      <c r="F92" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6">
+      <c r="A93" s="2">
+        <v>6222</v>
+      </c>
+      <c r="B93" t="str">
+        <f t="shared" si="4"/>
+        <v>62220000</v>
+      </c>
+      <c r="C93" t="str">
+        <f t="shared" si="5"/>
+        <v>n62220000</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E93" t="s">
+        <v>172</v>
+      </c>
+      <c r="F93" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6">
+      <c r="A94" s="2">
+        <v>639</v>
+      </c>
+      <c r="B94" t="str">
+        <f t="shared" si="4"/>
+        <v>63900000</v>
+      </c>
+      <c r="C94" t="str">
+        <f t="shared" si="5"/>
+        <v>n63900000</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="E94" t="s">
+        <v>172</v>
+      </c>
+      <c r="F94" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6">
+      <c r="A95" s="3">
+        <v>632</v>
+      </c>
+      <c r="B95" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>63200000</v>
+      </c>
+      <c r="C95" s="4" t="str">
+        <f t="shared" si="5"/>
+        <v>n63200000</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E95" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6">
+      <c r="A96" s="2">
+        <v>7</v>
+      </c>
+      <c r="B96" t="str">
+        <f t="shared" si="4"/>
+        <v>70000000</v>
+      </c>
+      <c r="C96" t="str">
+        <f t="shared" si="5"/>
+        <v>n70000000</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E96" t="s">
+        <v>174</v>
+      </c>
+      <c r="F96" t="s">
+        <v>174</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1" xr:uid="{853D7656-B308-4E3A-9467-98AD8F1F4D68}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Working on figures for vegetation model v1.0.5. Also, added notebook with dataframe pull for preliminary uncertainty analysis inputs.
</commit_message>
<xml_diff>
--- a/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
+++ b/src/LULUCF/LULUCF_state_node_lookup_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIS\git\AFOLU_GHG_flux_model\src\LULUCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B50FB4FA-4274-41B1-B8FD-9E495C0ECEFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4685BF5-E675-465A-95B2-54E3D07852D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-9795" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-225" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="v030_20250430" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">v040_20250713!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">v042_20250805!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">v102_20251027!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">v102_20251027!$A$1:$G$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="202">
   <si>
     <t>meaning</t>
   </si>
@@ -629,6 +629,27 @@
   </si>
   <si>
     <t>land_state</t>
+  </si>
+  <si>
+    <t>tall_veg_type</t>
+  </si>
+  <si>
+    <t>mangrove</t>
+  </si>
+  <si>
+    <t>oil_palm</t>
+  </si>
+  <si>
+    <t>non_oil_palm_planted_trees</t>
+  </si>
+  <si>
+    <t>natural_tree_cover</t>
+  </si>
+  <si>
+    <t>trees_in_other_land_covers</t>
+  </si>
+  <si>
+    <t>non_tall_vegetation</t>
   </si>
 </sst>
 </file>
@@ -688,7 +709,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -698,6 +719,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5547,18 +5569,19 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A7BB84B-4BF3-4978-BFCA-0C4F8A30C442}">
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="132.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="125.54296875" customWidth="1"/>
     <col min="5" max="5" width="15.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="30.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>193</v>
       </c>
@@ -5577,8 +5600,11 @@
       <c r="F1" s="1" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" s="2">
         <v>111</v>
       </c>
@@ -5599,8 +5625,11 @@
       <c r="F2" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="G2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" s="2">
         <v>112</v>
       </c>
@@ -5621,8 +5650,11 @@
       <c r="F3" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
+      <c r="G3" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" s="2">
         <v>122</v>
       </c>
@@ -5643,8 +5675,11 @@
       <c r="F4" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="G4" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" s="2">
         <v>123</v>
       </c>
@@ -5665,8 +5700,11 @@
       <c r="F5" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="G5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" s="2">
         <v>124</v>
       </c>
@@ -5687,8 +5725,11 @@
       <c r="F6" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="G6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" s="2">
         <v>125</v>
       </c>
@@ -5709,8 +5750,11 @@
       <c r="F7" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="G7" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" s="2">
         <v>126</v>
       </c>
@@ -5731,8 +5775,11 @@
       <c r="F8" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="G8" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9" s="2">
         <v>127</v>
       </c>
@@ -5753,8 +5800,11 @@
       <c r="F9" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="10" spans="1:6">
+      <c r="G9" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" s="2">
         <v>121</v>
       </c>
@@ -5775,8 +5825,11 @@
       <c r="F10" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
+      <c r="G10" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11" s="2">
         <v>131</v>
       </c>
@@ -5797,8 +5850,11 @@
       <c r="F11" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="12" spans="1:6">
+      <c r="G11" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
       <c r="A12" s="2">
         <v>132</v>
       </c>
@@ -5819,8 +5875,11 @@
       <c r="F12" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="13" spans="1:6">
+      <c r="G12" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
       <c r="A13" s="2">
         <v>100</v>
       </c>
@@ -5841,8 +5900,11 @@
       <c r="F13" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="14" spans="1:6">
+      <c r="G13" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
       <c r="A14" s="2">
         <v>101</v>
       </c>
@@ -5863,8 +5925,11 @@
       <c r="F14" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" s="4" customFormat="1">
+      <c r="G14" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" s="4" customFormat="1">
       <c r="A15" s="3">
         <v>102</v>
       </c>
@@ -5885,8 +5950,11 @@
       <c r="F15" s="4" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="16" spans="1:6">
+      <c r="G15" s="4" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
       <c r="A16" s="2">
         <v>211</v>
       </c>
@@ -5907,8 +5975,11 @@
       <c r="F16" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="17" spans="1:6">
+      <c r="G16" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
       <c r="A17" s="2">
         <v>212</v>
       </c>
@@ -5929,8 +6000,11 @@
       <c r="F17" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="18" spans="1:6">
+      <c r="G17" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
       <c r="A18" s="2">
         <v>221</v>
       </c>
@@ -5951,8 +6025,11 @@
       <c r="F18" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" s="4" customFormat="1">
+      <c r="G18" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" s="4" customFormat="1">
       <c r="A19" s="3">
         <v>222</v>
       </c>
@@ -5973,8 +6050,11 @@
       <c r="F19" s="4" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="20" spans="1:6">
+      <c r="G19" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
       <c r="A20" s="2">
         <v>3119</v>
       </c>
@@ -5995,8 +6075,11 @@
       <c r="F20" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="21" spans="1:6">
+      <c r="G20" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
       <c r="A21" s="2">
         <v>3112</v>
       </c>
@@ -6017,8 +6100,11 @@
       <c r="F21" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="22" spans="1:6">
+      <c r="G21" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
       <c r="A22" s="2">
         <v>312119</v>
       </c>
@@ -6039,8 +6125,11 @@
       <c r="F22" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="23" spans="1:6">
+      <c r="G22" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
       <c r="A23" s="2">
         <v>312112</v>
       </c>
@@ -6061,8 +6150,11 @@
       <c r="F23" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="24" spans="1:6">
+      <c r="G23" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
       <c r="A24" s="2">
         <v>312129</v>
       </c>
@@ -6083,8 +6175,11 @@
       <c r="F24" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="25" spans="1:6">
+      <c r="G24" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
       <c r="A25" s="2">
         <v>312122</v>
       </c>
@@ -6105,8 +6200,11 @@
       <c r="F25" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="26" spans="1:6">
+      <c r="G25" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
       <c r="A26" s="2">
         <v>312219</v>
       </c>
@@ -6127,8 +6225,11 @@
       <c r="F26" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="27" spans="1:6">
+      <c r="G26" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
       <c r="A27" s="2">
         <v>312212</v>
       </c>
@@ -6149,8 +6250,11 @@
       <c r="F27" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="28" spans="1:6">
+      <c r="G27" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
       <c r="A28" s="2">
         <v>312229</v>
       </c>
@@ -6171,8 +6275,11 @@
       <c r="F28" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="29" spans="1:6">
+      <c r="G28" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
       <c r="A29" s="2">
         <v>312222</v>
       </c>
@@ -6193,8 +6300,11 @@
       <c r="F29" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="30" spans="1:6">
+      <c r="G29" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
       <c r="A30" s="2">
         <v>312319</v>
       </c>
@@ -6215,8 +6325,11 @@
       <c r="F30" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="31" spans="1:6">
+      <c r="G30" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
       <c r="A31" s="2">
         <v>312312</v>
       </c>
@@ -6237,8 +6350,11 @@
       <c r="F31" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="32" spans="1:6">
+      <c r="G31" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
       <c r="A32" s="2">
         <v>312329</v>
       </c>
@@ -6259,8 +6375,11 @@
       <c r="F32" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="33" spans="1:6">
+      <c r="G32" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
       <c r="A33" s="2">
         <v>312322</v>
       </c>
@@ -6281,8 +6400,11 @@
       <c r="F33" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="34" spans="1:6">
+      <c r="G33" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
       <c r="A34" s="2">
         <v>312412</v>
       </c>
@@ -6303,8 +6425,11 @@
       <c r="F34" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="35" spans="1:6">
+      <c r="G34" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
       <c r="A35" s="2">
         <v>312422</v>
       </c>
@@ -6325,8 +6450,11 @@
       <c r="F35" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="36" spans="1:6">
+      <c r="G35" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" s="2">
         <v>32119</v>
       </c>
@@ -6347,8 +6475,11 @@
       <c r="F36" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="37" spans="1:6">
+      <c r="G36" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" s="2">
         <v>32112</v>
       </c>
@@ -6369,8 +6500,11 @@
       <c r="F37" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="38" spans="1:6">
+      <c r="G37" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
       <c r="A38" s="2">
         <v>321219</v>
       </c>
@@ -6391,8 +6525,11 @@
       <c r="F38" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="39" spans="1:6">
+      <c r="G38" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" s="2">
         <v>321212</v>
       </c>
@@ -6413,8 +6550,11 @@
       <c r="F39" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="40" spans="1:6">
+      <c r="G39" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
       <c r="A40" s="2">
         <v>321229</v>
       </c>
@@ -6435,8 +6575,11 @@
       <c r="F40" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="41" spans="1:6">
+      <c r="G40" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
       <c r="A41" s="2">
         <v>321222</v>
       </c>
@@ -6457,8 +6600,11 @@
       <c r="F41" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="42" spans="1:6">
+      <c r="G41" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
       <c r="A42" s="2">
         <v>32139</v>
       </c>
@@ -6479,8 +6625,11 @@
       <c r="F42" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="43" spans="1:6">
+      <c r="G42" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
       <c r="A43" s="2">
         <v>32132</v>
       </c>
@@ -6501,8 +6650,11 @@
       <c r="F43" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="44" spans="1:6">
+      <c r="G43" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
       <c r="A44" s="2">
         <v>32142</v>
       </c>
@@ -6523,8 +6675,11 @@
       <c r="F44" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="45" spans="1:6">
+      <c r="G44" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
       <c r="A45" s="2">
         <v>32219</v>
       </c>
@@ -6545,8 +6700,11 @@
       <c r="F45" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="46" spans="1:6">
+      <c r="G45" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
       <c r="A46" s="2">
         <v>32212</v>
       </c>
@@ -6567,8 +6725,11 @@
       <c r="F46" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="47" spans="1:6">
+      <c r="G46" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
       <c r="A47" s="2">
         <v>32229</v>
       </c>
@@ -6589,8 +6750,11 @@
       <c r="F47" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="48" spans="1:6">
+      <c r="G47" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
       <c r="A48" s="2">
         <v>32222</v>
       </c>
@@ -6611,8 +6775,11 @@
       <c r="F48" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="49" spans="1:6">
+      <c r="G48" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
       <c r="A49" s="2">
         <v>32239</v>
       </c>
@@ -6633,8 +6800,11 @@
       <c r="F49" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="50" spans="1:6">
+      <c r="G49" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
       <c r="A50" s="2">
         <v>32232</v>
       </c>
@@ -6655,8 +6825,11 @@
       <c r="F50" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" s="4" customFormat="1">
+      <c r="G50" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" s="4" customFormat="1">
       <c r="A51" s="3">
         <v>32242</v>
       </c>
@@ -6677,8 +6850,11 @@
       <c r="F51" s="4" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="52" spans="1:6">
+      <c r="G51" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
       <c r="A52" s="2">
         <v>419</v>
       </c>
@@ -6699,8 +6875,11 @@
       <c r="F52" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="53" spans="1:6">
+      <c r="G52" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
       <c r="A53" s="2">
         <v>412</v>
       </c>
@@ -6721,8 +6900,11 @@
       <c r="F53" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="54" spans="1:6">
+      <c r="G53" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
       <c r="A54" s="2">
         <v>4211119</v>
       </c>
@@ -6743,8 +6925,11 @@
       <c r="F54" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="55" spans="1:6">
+      <c r="G54" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
       <c r="A55" s="2">
         <v>4211112</v>
       </c>
@@ -6765,8 +6950,11 @@
       <c r="F55" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="56" spans="1:6">
+      <c r="G55" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
       <c r="A56" s="2">
         <v>4211129</v>
       </c>
@@ -6787,8 +6975,11 @@
       <c r="F56" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="57" spans="1:6">
+      <c r="G56" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
       <c r="A57" s="2">
         <v>4211122</v>
       </c>
@@ -6809,8 +7000,11 @@
       <c r="F57" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="58" spans="1:6">
+      <c r="G57" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
       <c r="A58" s="2">
         <v>4211219</v>
       </c>
@@ -6831,8 +7025,11 @@
       <c r="F58" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="59" spans="1:6">
+      <c r="G58" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
       <c r="A59" s="2">
         <v>4211212</v>
       </c>
@@ -6853,8 +7050,11 @@
       <c r="F59" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="60" spans="1:6">
+      <c r="G59" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
       <c r="A60" s="2">
         <v>4211229</v>
       </c>
@@ -6875,8 +7075,11 @@
       <c r="F60" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="61" spans="1:6">
+      <c r="G60" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
       <c r="A61" s="2">
         <v>4211222</v>
       </c>
@@ -6897,8 +7100,11 @@
       <c r="F61" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="62" spans="1:6">
+      <c r="G61" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7">
       <c r="A62" s="2">
         <v>4212119</v>
       </c>
@@ -6919,8 +7125,11 @@
       <c r="F62" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="63" spans="1:6">
+      <c r="G62" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7">
       <c r="A63" s="2">
         <v>4212112</v>
       </c>
@@ -6941,8 +7150,11 @@
       <c r="F63" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="64" spans="1:6">
+      <c r="G63" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7">
       <c r="A64" s="2">
         <v>4212129</v>
       </c>
@@ -6963,8 +7175,11 @@
       <c r="F64" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="65" spans="1:6">
+      <c r="G64" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7">
       <c r="A65" s="2">
         <v>4212122</v>
       </c>
@@ -6985,8 +7200,11 @@
       <c r="F65" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="66" spans="1:6">
+      <c r="G65" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7">
       <c r="A66" s="2">
         <v>4212219</v>
       </c>
@@ -7007,8 +7225,11 @@
       <c r="F66" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="67" spans="1:6">
+      <c r="G66" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7">
       <c r="A67" s="2">
         <v>4212212</v>
       </c>
@@ -7029,8 +7250,11 @@
       <c r="F67" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="68" spans="1:6">
+      <c r="G67" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7">
       <c r="A68" s="2">
         <v>4212229</v>
       </c>
@@ -7051,8 +7275,11 @@
       <c r="F68" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="69" spans="1:6">
+      <c r="G68" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7">
       <c r="A69" s="2">
         <v>4212222</v>
       </c>
@@ -7073,8 +7300,11 @@
       <c r="F69" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="70" spans="1:6">
+      <c r="G69" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7">
       <c r="A70" s="2">
         <v>422119</v>
       </c>
@@ -7095,8 +7325,11 @@
       <c r="F70" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="71" spans="1:6">
+      <c r="G70" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7">
       <c r="A71" s="2">
         <v>422112</v>
       </c>
@@ -7117,8 +7350,11 @@
       <c r="F71" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="72" spans="1:6">
+      <c r="G71" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7">
       <c r="A72" s="2">
         <v>422129</v>
       </c>
@@ -7139,8 +7375,11 @@
       <c r="F72" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="73" spans="1:6">
+      <c r="G72" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7">
       <c r="A73" s="2">
         <v>422122</v>
       </c>
@@ -7161,8 +7400,11 @@
       <c r="F73" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="74" spans="1:6">
+      <c r="G73" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7">
       <c r="A74" s="2">
         <v>4222119</v>
       </c>
@@ -7183,8 +7425,11 @@
       <c r="F74" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="75" spans="1:6">
+      <c r="G74" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7">
       <c r="A75" s="2">
         <v>4222112</v>
       </c>
@@ -7205,8 +7450,11 @@
       <c r="F75" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="76" spans="1:6">
+      <c r="G75" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7">
       <c r="A76" s="2">
         <v>42221219</v>
       </c>
@@ -7227,8 +7475,11 @@
       <c r="F76" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="77" spans="1:6">
+      <c r="G76" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7">
       <c r="A77" s="2">
         <v>42221212</v>
       </c>
@@ -7249,8 +7500,11 @@
       <c r="F77" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="78" spans="1:6">
+      <c r="G77" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7">
       <c r="A78" s="2">
         <v>42221229</v>
       </c>
@@ -7271,8 +7525,11 @@
       <c r="F78" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="79" spans="1:6">
+      <c r="G78" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7">
       <c r="A79" s="2">
         <v>42221222</v>
       </c>
@@ -7293,8 +7550,11 @@
       <c r="F79" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="80" spans="1:6">
+      <c r="G79" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7">
       <c r="A80" s="2">
         <v>422229</v>
       </c>
@@ -7315,8 +7575,11 @@
       <c r="F80" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="81" spans="1:6">
+      <c r="G80" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" s="4" customFormat="1">
       <c r="A81" s="3">
         <v>422222</v>
       </c>
@@ -7337,8 +7600,11 @@
       <c r="F81" s="4" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="82" spans="1:6">
+      <c r="G81" s="4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7">
       <c r="A82" s="2">
         <v>51</v>
       </c>
@@ -7359,8 +7625,11 @@
       <c r="F82" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="83" spans="1:6">
+      <c r="G82" s="5" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7">
       <c r="A83" s="2">
         <v>5219</v>
       </c>
@@ -7381,8 +7650,11 @@
       <c r="F83" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="84" spans="1:6">
+      <c r="G83" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7">
       <c r="A84" s="2">
         <v>5212</v>
       </c>
@@ -7403,8 +7675,11 @@
       <c r="F84" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="85" spans="1:6">
+      <c r="G84" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7">
       <c r="A85" s="2">
         <v>5222</v>
       </c>
@@ -7425,8 +7700,11 @@
       <c r="F85" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="86" spans="1:6">
+      <c r="G85" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7">
       <c r="A86" s="2">
         <v>5239</v>
       </c>
@@ -7447,8 +7725,11 @@
       <c r="F86" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="87" spans="1:6">
+      <c r="G86" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7">
       <c r="A87" s="2">
         <v>5232</v>
       </c>
@@ -7469,8 +7750,11 @@
       <c r="F87" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="88" spans="1:6">
+      <c r="G87" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7">
       <c r="A88" s="2">
         <v>539</v>
       </c>
@@ -7491,8 +7775,11 @@
       <c r="F88" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="89" spans="1:6">
+      <c r="G88" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" s="4" customFormat="1">
       <c r="A89" s="3">
         <v>532</v>
       </c>
@@ -7513,8 +7800,11 @@
       <c r="F89" s="4" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="90" spans="1:6">
+      <c r="G89" s="4" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7">
       <c r="A90" s="2">
         <v>61</v>
       </c>
@@ -7535,8 +7825,11 @@
       <c r="F90" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="91" spans="1:6">
+      <c r="G90" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7">
       <c r="A91" s="2">
         <v>6212</v>
       </c>
@@ -7557,8 +7850,11 @@
       <c r="F91" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="92" spans="1:6">
+      <c r="G91" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7">
       <c r="A92" s="2">
         <v>6229</v>
       </c>
@@ -7579,8 +7875,11 @@
       <c r="F92" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="93" spans="1:6">
+      <c r="G92" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7">
       <c r="A93" s="2">
         <v>6222</v>
       </c>
@@ -7601,8 +7900,11 @@
       <c r="F93" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="94" spans="1:6">
+      <c r="G93" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7">
       <c r="A94" s="2">
         <v>639</v>
       </c>
@@ -7623,8 +7925,11 @@
       <c r="F94" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="95" spans="1:6">
+      <c r="G94" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" s="4" customFormat="1">
       <c r="A95" s="3">
         <v>632</v>
       </c>
@@ -7645,8 +7950,11 @@
       <c r="F95" s="4" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="96" spans="1:6">
+      <c r="G95" s="4" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7">
       <c r="A96" s="2">
         <v>7</v>
       </c>
@@ -7667,9 +7975,12 @@
       <c r="F96" t="s">
         <v>174</v>
       </c>
+      <c r="G96" t="s">
+        <v>201</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{853D7656-B308-4E3A-9467-98AD8F1F4D68}"/>
+  <autoFilter ref="A1:G1" xr:uid="{6A7BB84B-4BF3-4978-BFCA-0C4F8A30C442}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>